<commit_message>
B&N rev8 WIP: back-check FAIL fixes (S-12, RFI texts, Tek screws, 16 ga wire), family order fix, skill v80o R80e.29
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01UQBQT8jCVU6KW8QmKhZS83
</commit_message>
<xml_diff>
--- a/cache_proyectos/barnes_noble/takeoff_work/etapas/8_excel/Barnes_Noble_ColoradoSprings_Takeoff_FINAL_rev8.xlsx
+++ b/cache_proyectos/barnes_noble/takeoff_work/etapas/8_excel/Barnes_Noble_ColoradoSprings_Takeoff_FINAL_rev8.xlsx
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1036" uniqueCount="707">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1044" uniqueCount="711">
   <si>
     <t xml:space="preserve">Barnes &amp; Noble - Colorado Springs, CO (3173 Cinema Point)   |   METAL FRAMING &amp; DRYWALL TAKEOFF</t>
   </si>
@@ -91,7 +91,7 @@
     <t xml:space="preserve">n/a</t>
   </si>
   <si>
-    <t xml:space="preserve">Project value (canon constants).</t>
+    <t xml:space="preserve">Project value (not used in this take-off: heights are per wall in the Partition Takeoff).</t>
   </si>
   <si>
     <t xml:space="preserve">B.O. Deck (ft)</t>
@@ -1087,7 +1087,7 @@
     <t xml:space="preserve">Hanger wire</t>
   </si>
   <si>
-    <t xml:space="preserve">N/SHEET: 5/A-121, 1/A-121 | Breakdown [DERIVED]: Women's Restroom 109 144 + Men's Restroom 108 144 + Cafe 103 - 11'-6" GWB band 243 + Cafe 103 - 9'-0" GWB band 192 + Cafe Seating Area 102 - GWB cloud 715 + Grab &amp; Go 107.5 + HANGERS-FIXTURES-5-A121 401 + SPLAY-WIRES-5-A121 743.29 + SEISMIC-VERTICAL-WIRE-5-A121 131.42 = 2,821.21 LF (hangers @ 48" O.C. x drop to deck per room)</t>
+    <t xml:space="preserve">N/SHEET: 5/A-121, 1/A-121 | Breakdown [DERIVED]: Women's Restroom 109 144 + Men's Restroom 108 144 + Cafe 103 - 11'-6" GWB band 243 + Cafe 103 - 9'-0" GWB band 192 + Cafe Seating Area 102 - GWB cloud 715 + Grab &amp; Go 107.5 + HANGERS-FIXTURES-5-A121 401 + SPLAY-WIRES-5-A121 743.29 = 2,689.79 LF (hangers @ 48" O.C. x drop to deck per room)</t>
   </si>
   <si>
     <t xml:space="preserve">Blocking FRT / 2X FRT wood</t>
@@ -1150,7 +1150,19 @@
     <t xml:space="preserve">#8 pan head self-tapping screws, relief channel to structure (8/A-410)</t>
   </si>
   <si>
-    <t xml:space="preserve">N/SHEET: 8/A-410 | Breakdown [DERIVED]: PAN-HEAD-8-A410 291 = 291 PCS | 8/A-410 "CONTINUOUS 20 GA. X 2" MIN DEEP RELIEF CHANNEL - ANCHOR TO STEEL PLATE WITH #8 PAN HEAD SELF TAPPING SCREWS AT 24" O.C. AND 6" FROM ENDS": sum(ROUNDUP(L / 2) + 1) over 32 runs to structure (479.85 LF) = 291 pcs (Paso 12 C7-03; note 8.C X-EDNI = alternative in RFI-51)</t>
+    <t xml:space="preserve">N/SHEET: 8/A-410 | Breakdown [DERIVED]: PAN-HEAD-8-A410 291 = 291 PCS | 8/A-410 "CONTINUOUS 20 GA. X 2" MIN DEEP RELIEF CHANNEL - ANCHOR TO STEEL PLATE WITH #8 PAN HEAD SELF TAPPING SCREWS AT 24" O.C. AND 6" FROM ENDS": sum(ROUNDUP(L / 2) + 1) over 32 runs to structure (479.85 LF) = 291 pcs (rev7 plan check C7-03; note 8.C X-EDNI = alternative in RFI-51)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">#8 Tek screws at clip angles ((4) per clip, 5/A-410; 7/A-210)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">N/SHEET: 5/A-410, 7/A-210 | Breakdown [DERIVED]: TEK-SCREWS-CLIPS 10,088 = 10,088 PCS | 5/A-410 "2" x 2" 16 GA. CLIP ANGLE ... (4) TEK SCREWS": 2518 clips x 4 = 10072 + 7/A-210 "(4) #10-16 SCREWS": 4 clips x 4 = 16; total 10088 pcs</t>
+  </si>
+  <si>
+    <t xml:space="preserve">16 ga wire at seismic brace points (5/A-121)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">N/SHEET: 5/A-121 | Breakdown [DERIVED]: SEISMIC-VERTICAL-WIRE-5-A121 131.42 = 131.42 LF | 5/A-121 "16 GA. WIRE 12'-0\" O.C. EACH WAY AND WITHIN 6'-0\" OF EACH WALL" vertical wire at each brace point: groups Women's 1 x drop 16.0; Men's 1 x drop 16.0; Cafe 11'-6" band 1 x drop 13.5; Cafe 9'-0" band 1 x drop 16.0; Cafe cloud 4 x drop 13.0; Grab &amp; Go 1 x drop 17.917 -&gt; sum(groups x drop) = 131.42 LF (conservative - RFI-38) - rev7 plan check C7-01: the 1-5/8" x 16 ga metal joist framing @ 48" O.C. on 5/A-121 is the horizontal carrying member (no post drawn)</t>
   </si>
   <si>
     <t xml:space="preserve">P.A.F. 3/16" x 3/8" at cross member ends (8/A-410)</t>
@@ -1162,7 +1174,7 @@
     <t xml:space="preserve">5/8" cement board (tile base)</t>
   </si>
   <si>
-    <t xml:space="preserve">N/SHEET: 22/A-201 | Breakdown [DERIVED]: RESTROOM-BASE-CEMENT 50.04 = 50.04 SF | 5/8" CEMENT BOARD BASE 1'-2" (22/A-201; A-001A Div 09 J.2): W2-05 7.51 + W2-06.1 6.92 + W2-06.2 2.23 + W2-06.3 2.41 + W2-06.3 2.46 + W2-06.4 2.23 + W2-06.5 6.88 + W2-07 7.51 + W5-01 5.7 + W5-01 5.7 = 49.55 LF - doors 8, 9 (6.66) = 42.89 LF x 1'-2" = 50.04 SF - Paso 12 C-03</t>
+    <t xml:space="preserve">N/SHEET: 22/A-201 | Breakdown [DERIVED]: RESTROOM-BASE-CEMENT 50.04 = 50.04 SF | 5/8" CEMENT BOARD BASE 1'-2" (22/A-201; A-001A Div 09 J.2): W2-05 7.51 + W2-06.1 6.92 + W2-06.2 2.23 + W2-06.3 2.41 + W2-06.3 2.46 + W2-06.4 2.23 + W2-06.5 6.88 + W2-07 7.51 + W5-01 5.7 + W5-01 5.7 = 49.55 LF - doors 8, 9 (6.66) = 42.89 LF x 1'-2" = 50.04 SF - rev7 plan check C-03</t>
   </si>
   <si>
     <t xml:space="preserve">Plywood screws #10-24 x 1-1/4" Teks/3 (A-410 note 8.D)</t>
@@ -1282,7 +1294,7 @@
     <t xml:space="preserve">Drywall screws #7 x 1-1/4" Type S bugle head (board on 25/20 ga studs)</t>
   </si>
   <si>
-    <t xml:space="preserve">[DERIVED] N/SHEET: A-410, A-001A | Inputs!B20 (Drywall screws per SF of board = 1.2) x 5335.22 SF of board</t>
+    <t xml:space="preserve">[DERIVED] N/SHEET: A-410, A-001A | Inputs!B20 (Drywall screws per SF of board = 1.2) x 5058.29 SF of board</t>
   </si>
   <si>
     <t xml:space="preserve">Framing screws #8-18 x 1/2" pan head (25/20 ga studs)</t>
@@ -1342,7 +1354,7 @@
     <t xml:space="preserve">Type S-12 drywall screws #6 x 1-1/4" (board on 18/16/14 ga studs)</t>
   </si>
   <si>
-    <t xml:space="preserve">[DERIVED] N/SHEET: A-410 | 1.2 x 10866.66 SF of board on the 18/16/14 ga walls (C-F, C-H2a, C-H2b, W2-01, W2-02, W2-03, W2-04, W2-05, W2-06.1, W2-06.2, W2-06.3, W2-06.4, W2-06.5, W2-07, W2-08, W2-09) = 13039.99</t>
+    <t xml:space="preserve">[DERIVED] N/SHEET: A-410 | 1.2 x 11143.59 SF of board on the 18/16/14 ga walls (C-F, C-H2a, C-H2b, W2-01, W2-02, W2-03, W2-04, W2-05, W2-06.1, W2-06.2, W2-06.3, W2-06.4, W2-06.5, W2-07, W2-08, W2-09) = 13372.31</t>
   </si>
   <si>
     <t xml:space="preserve">RFI</t>
@@ -1357,7 +1369,7 @@
     <t xml:space="preserve">RFI-ACC-slab-pins</t>
   </si>
   <si>
-    <t xml:space="preserve">slab pins: pin spacing: carried one pin every 8.0" (A-410 Partition Notes 8.F "0.145" DIA. HILTI X-DNI FASTENER, 1" MIN. LENGTH, 2 ROWS AT 16" O.C." (printed, conservative) vs 9/A-410 "0.177 D); alternatives: one row @ 16" / one row @ 24" (v80o: printed spacings, BE-19)</t>
+    <t xml:space="preserve">slab pins: pin spacing: carried one pin every 8.0" (A-410 note 8.F X-DNI 2 rows @ 16" O.C. (printed, conservative); 9/A-410 0.177" PAF @ 24" = alternative); alternatives: one row @ 16" / one row @ 24"</t>
   </si>
   <si>
     <t xml:space="preserve">16in: -480.46 pcs; 24in: -640.61 pcs</t>
@@ -1375,7 +1387,7 @@
     <t xml:space="preserve">RFI-01</t>
   </si>
   <si>
-    <t xml:space="preserve">CLOSED - estimator decision 2026-10-24 (rev1): perimeter walls types 1 / 1A / 1B / 1C are EXISTING (1/DM-101 legend solid = to remain + key note 3 "EXTERIOR WALL PATCH AND REPAIR AS REQUIRED TO MAINTAIN EXISTING FIRE RATING"; A-101 Construction Legend "EXISTING EXTERIOR WALL" / "EXISTING PARTITION"; A-002 "PERIMETER STUDS, INSULATION, VAPOR BARRIER F/I BY LL"). Perimeter framing (studs, track, bracing, 1B sheathing) EXCLUDED. Interior face patch &amp; repair (1/DM-101 key note 3, A-101 C5) = ALLOWANCE, amount: $ ________ (blank, estimator to fill). rev2 (estimator decision 2026-10-25): break room kitchenette W.R. on existing EXT-07 (6/A-412, 7/A-412) is INSIDE this patch &amp; repair allowance; allowance amount stays BLANK (decided). Paso 12 (rev7): A-410 types 1, 1A, 1B, 1C label the interior board "5/8" GYP BD BY FUTURE TENANT": EXCLUDED with that citation, consistent with this decision. A-413 7/8A general note "IF SHELVING IS TO BE INSTALLED ON EXISTING WALL, G.C. IS TO REMOVE AND REPLACE GYP. BOARD AS REQUIRED FOR INSTALLATION OF WOOD BLOCKING": inside this patch &amp; repair allowance.</t>
+    <t xml:space="preserve">CLOSED - estimator decision 2026-10-24 (rev1): perimeter walls types 1 / 1A / 1B / 1C are EXISTING (1/DM-101 legend solid = to remain + key note 3 "EXTERIOR WALL PATCH AND REPAIR AS REQUIRED TO MAINTAIN EXISTING FIRE RATING"; A-101 Construction Legend "EXISTING EXTERIOR WALL" / "EXISTING PARTITION"; A-002 "PERIMETER STUDS, INSULATION, VAPOR BARRIER F/I BY LL"). Perimeter framing (studs, track, bracing, 1B sheathing) EXCLUDED. Interior face patch &amp; repair (1/DM-101 key note 3, A-101 C5) = ALLOWANCE, amount: $ ________ (blank, estimator to fill). rev2 (estimator decision 2026-10-25): break room kitchenette W.R. on existing EXT-07 (6/A-412, 7/A-412) is INSIDE this patch &amp; repair allowance; allowance amount stays BLANK (decided). Plan check (rev7): A-410 types 1, 1A, 1B, 1C label the interior board "5/8" GYP BD BY FUTURE TENANT": EXCLUDED with that citation, consistent with this decision. A-413 7/8A general note "IF SHELVING IS TO BE INSTALLED ON EXISTING WALL, G.C. IS TO REMOVE AND REPLACE GYP. BOARD AS REQUIRED FOR INSTALLATION OF WOOD BLOCKING": inside this patch &amp; repair allowance.</t>
   </si>
   <si>
     <t xml:space="preserve">Applied: - 417.43 LF of perimeter walls (17 walls); 3-5/8" stud 16,812.96 -&gt; 10,120.39 LF; 8" stud 2,332.99 -&gt; 0; 1/2" exterior sheathing 2,469.22 -&gt; 0 SF; bottom / top track 1,051.87 -&gt; 634.44 LF each; bracing 5,230.74 -&gt; 2,827.81 LF. Allowance: blank.; board by future tenant on the existing perimeter (A-410 types 1 / 1A / 1B / 1C): upper bound 417.43 LF x 25.0 = 10,436 SF 5/8" Type X if it were ever in our scope.</t>
@@ -1393,7 +1405,7 @@
     <t xml:space="preserve">RFI-03</t>
   </si>
   <si>
-    <t xml:space="preserve">B.O. deck is V.I.F. and sloped: 24'-0" (2/A-400B) to 25'-7" (2/A-400A); walls to deck loaded at 25'-0" (1/A-400A, 1/A-400B), east facade 25'-7", west 24'-0". Paso 12 (rev7): the elevations also print 21'-9" V.I.F. at the right end of 2/A-400A and 23'-8" V.I.F. on A-400B (joists sloping): the B.O. deck range is wider than 24'-0" to 25'-7".</t>
+    <t xml:space="preserve">B.O. deck is V.I.F. and sloped: 24'-0" (2/A-400B) to 25'-7" (2/A-400A); walls to deck loaded at 25'-0" (1/A-400A, 1/A-400B), east facade 25'-7", west 24'-0". Plan check (rev7): the elevations also print 21'-9" V.I.F. at the right end of 2/A-400A and 23'-8" V.I.F. on A-400B (joists sloping): the B.O. deck range is wider than 24'-0" to 25'-7".</t>
   </si>
   <si>
     <t xml:space="preserve">Each 1 ft of deck height = 414.54 LF of studs-to-deck walls x 1 ft (studs, board where to deck, bracing rows)</t>
@@ -1402,10 +1414,10 @@
     <t xml:space="preserve">RFI-04</t>
   </si>
   <si>
-    <t xml:space="preserve">CLOSED - Review Item rev3 (estimator decision 2026-10-26): type 2 &gt; 22 ft: 3-5/8" 14 ga SJ + diagonal braces @ 32" O.C. to structure (3/A-410 Top Track Detail "PROVIDE DIAGONAL BRACING AT 32" O.C. TO STRUCTURE ABOVE (TYP.)"); brace member / length not printed - estimator choice 3-5/8" 20 ga stud x 4 ft at 45 deg. Paso 12 (rev7): same precedent applied to the Cafe 3-5/8" walls to deck (C-H2a, C-H2b, C-F): 14 ga SJ + 11 diagonal braces = 44.0 LF.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Applied: 117 braces x 4.0 ft = 468.0 LF (type 2) + 44.0 LF (Cafe) 3-5/8" 20 ga stud (member and length = estimator choice). Citation history: rev0-rev2 cited the partition type 3 section, rev3-rev6 cited 8/A-410 (that bubble is the Typ. Connection Detail); the Top Track Detail is bubble 3/A-410 (Paso 12 C-07).</t>
+    <t xml:space="preserve">CLOSED - Review Item rev3 (estimator decision 2026-10-26): type 2 &gt; 22 ft: 3-5/8" 14 ga SJ + diagonal braces @ 32" O.C. to structure (3/A-410 Top Track Detail "PROVIDE DIAGONAL BRACING AT 32" O.C. TO STRUCTURE ABOVE (TYP.)"); brace member / length not printed - estimator choice 3-5/8" 20 ga stud x 4 ft at 45 deg. Plan check (rev7): same precedent applied to the Cafe 3-5/8" walls to deck (C-H2a, C-H2b, C-F): 14 ga SJ + 11 diagonal braces = 44.0 LF.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Applied: 117 braces x 4.0 ft = 468.0 LF (type 2) + 44.0 LF (Cafe) 3-5/8" 20 ga stud (member and length = estimator choice). Citation history: rev0-rev2 cited the partition type 3 section, rev3-rev6 cited 8/A-410 (that bubble is the Typ. Connection Detail); the Top Track Detail is bubble 3/A-410 (rev7 plan check C-07).</t>
   </si>
   <si>
     <t xml:space="preserve">RFI-05</t>
@@ -1468,7 +1480,7 @@
     <t xml:space="preserve">RFI-12</t>
   </si>
   <si>
-    <t xml:space="preserve">CLOSED (base) / OPEN (installer of tile) - Paso 12 (rev7): 22/A-201 Tile Base Detail prints "5/8" CEMENT BOARD" with "1'-2" CEMENT BOARD BASE" and 5/8" W.R. GYP. BD. above (A-001A Div 09 J.2). Corridor 110 wall tile (A-510) backer: not detailed.</t>
+    <t xml:space="preserve">CLOSED (base) / OPEN (installer of tile) - Plan check (rev7): 22/A-201 Tile Base Detail prints "5/8" CEMENT BOARD" with "1'-2" CEMENT BOARD BASE" and 5/8" W.R. GYP. BD. above (A-001A Div 09 J.2). Corridor 110 wall tile (A-510) backer: not detailed.</t>
   </si>
   <si>
     <t xml:space="preserve">Applied: + 50.04 SF cement board base on the restroom faces of new walls and the same SF out of W.R. Open: Corridor 110 wall tile backer - each 1 ft of tile height = 93.44 SF cement board instead of Type X.</t>
@@ -1477,7 +1489,7 @@
     <t xml:space="preserve">RFI-13</t>
   </si>
   <si>
-    <t xml:space="preserve">FRP-1 (A-510): Cafe Work Room 104 FRP-1 full height to the 10'-0" ceiling (1-4/A-226B); Janitor 107 FRP-1 to 96" A.F.F. (A-131) / 8'-0" (9-12/A-200). Who furnishes / installs the FRP is not defined (A-002). Substrate: E/A-221 and G/A-221 call 5/8" FRT plywood on the Work Room faces; 3/A-225 draws a dotted (board) fill - conflict. Not carried - Paso 12 (rev7): heights corrected.</t>
+    <t xml:space="preserve">FRP-1 (A-510): Cafe Work Room 104 FRP-1 full height to the 10'-0" ceiling (1-4/A-226B); Janitor 107 FRP-1 to 96" A.F.F. (A-131) / 8'-0" (9-12/A-200). Who furnishes / installs the FRP is not defined (A-002). Substrate: E/A-221 and G/A-221 call 5/8" FRT plywood on the Work Room faces; 3/A-225 draws a dotted (board) fill - conflict. Not carried - Plan check (rev7): heights corrected.</t>
   </si>
   <si>
     <t xml:space="preserve">If FRP is in our scope: Cafe Work Room 87.52 LF x 10.0 = 875.20 SF + Janitor 19.43 LF x 8.0 = 155.44 SF = 1,030.64 SF FRP-1 gross (doors not deducted) + PVC trim (J-mold, inside corners).</t>
@@ -1609,7 +1621,7 @@
     <t xml:space="preserve">Types 3 and 4 base anchorage: 3/A-410, 4/A-410 and A/A-410 draw a moment clip at the stud base with Hilti Kwik HUS-EZ anchors; spacing not printed separately. Not carried (expansion anchors 0).</t>
   </si>
   <si>
-    <t xml:space="preserve">If one clip per stud: + 162 moment clips (type 3 = 40 studs, type 4 = 122 studs, studs_out) + 324 Kwik HUS-EZ 1/4" x 1-5/8" (2 per clip)</t>
+    <t xml:space="preserve">If one clip per stud: + 162 moment clips (type 3 = 40 studs, type 4 = 122 studs, per-wall stud count) + 324 Kwik HUS-EZ 1/4" x 1-5/8" (2 per clip)</t>
   </si>
   <si>
     <t xml:space="preserve">RFI-29</t>
@@ -1660,7 +1672,7 @@
     <t xml:space="preserve">RFI-34</t>
   </si>
   <si>
-    <t xml:space="preserve">CLOSED - Paso 12 (rev7): T.O. WD-1 at the Grab &amp; Go header = 15'-0" (5/A-226A 11'-0" + 4'-0" WD-1; 6/A-226A 15'-0"). 3/A-221: 5/8" FRT plywood full face, 5/8" GWB over it above T.O. WD-1.</t>
+    <t xml:space="preserve">CLOSED - Plan check (rev7): T.O. WD-1 at the Grab &amp; Go header = 15'-0" (5/A-226A 11'-0" + 4'-0" WD-1; 6/A-226A 15'-0"). 3/A-221: 5/8" FRT plywood full face, 5/8" GWB over it above T.O. WD-1.</t>
   </si>
   <si>
     <t xml:space="preserve">Applied: + 6.167 x 10.0 = 61.67 SF 5/8" Type X (15'-0" to deck); FRT plywood unchanged (110.49 SF).</t>
@@ -1669,7 +1681,7 @@
     <t xml:space="preserve">RFI-35</t>
   </si>
   <si>
-    <t xml:space="preserve">3/A-410 Top Track Detail "METAL STUD/TRACK FIRE STOP AT CEILING LINE, TYP." (rev5-rev6 cited 8/A-410, which is the Typ. Connection Detail - Paso 12 C-07): applied to every full-height wall with a ceiling on at least one face (1/A-121); carried; confirm with the GC.</t>
+    <t xml:space="preserve">3/A-410 Top Track Detail "METAL STUD/TRACK FIRE STOP AT CEILING LINE, TYP." (rev5-rev6 cited 8/A-410, which is the Typ. Connection Detail - rev7 plan check C-07): applied to every full-height wall with a ceiling on at least one face (1/A-121); carried; confirm with the GC.</t>
   </si>
   <si>
     <t xml:space="preserve">Carried per wall (Material Summary breakdown) = 264.21 LF; if not required: minus that LF.</t>
@@ -1696,10 +1708,10 @@
     <t xml:space="preserve">RFI-38</t>
   </si>
   <si>
-    <t xml:space="preserve">Ceiling seismic bracing: A-121 Ceiling Notes 1 "SEE A-420 DRAWINGS REGARDING CEILING BRACING" - A-420 is not in the set; 5/A-121 draws splay wires @ 12'-0" O.C. each way and a 1-5/8" x 16 ga metal joist post; A-002 Div 10 "SEISMIC BRACING" F/I by the tenant contractor. Carried conservatively on the GWB suspended ceilings.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Carried: splay wires 743.29 LF + vertical 16 ga wire at each brace point 131.42 LF (both in the hanger wire row); the 1-5/8" x 16 ga metal joist framing @ 48" on 5/A-121 is the horizontal carrying member (no post) - Paso 12 2nd pass (rev8): C7-01. If not required: minus both.</t>
+    <t xml:space="preserve">Ceiling seismic bracing: A-121 Ceiling Notes 1 "SEE A-420 DRAWINGS REGARDING CEILING BRACING" - A-420 is not in the set; 5/A-121 draws splay wires and a 16 ga wire @ 12'-0" O.C. each way at each brace point (the 1-5/8" x 16 ga metal joist framing @ 48" is the horizontal carrying member); A-002 Div 10 "SEISMIC BRACING" F/I by the tenant contractor. Carried conservatively on the GWB suspended ceilings.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Carried: splay wires 743.29 LF (hanger wire row) + vertical 16 ga wire at each brace point 131.42 LF (16 ga wire row); the 1-5/8" x 16 ga metal joist framing @ 48" on 5/A-121 is the horizontal carrying member (no post) - Plan check (rev8): C7-01. If not required: minus both.</t>
   </si>
   <si>
     <t xml:space="preserve">RFI-39</t>
@@ -1768,7 +1780,7 @@
     <t xml:space="preserve">RFI-46</t>
   </si>
   <si>
-    <t xml:space="preserve">F/A-221 "3 5/8" METAL STUDS @ 16" O.C. TO BOTTOM OF NESTED STUD BRACING": the nested stud bracing member is not drawn; studs carried to deck (estimator decision RI 7). Paso 12 2nd pass (rev8): the same phrase is printed on the partition types 3 and 4 (3/A-410, 4/A-410): nested stud at the top of each wall.</t>
+    <t xml:space="preserve">F/A-221 "3 5/8" METAL STUDS @ 16" O.C. TO BOTTOM OF NESTED STUD BRACING": the nested stud bracing member is not drawn; studs carried to deck (estimator decision RI 7). Plan check (rev8): the same phrase is printed on the partition types 3 and 4 (3/A-410, 4/A-410): nested stud at the top of each wall.</t>
   </si>
   <si>
     <t xml:space="preserve">Carried 6.52 LF (F) + 122.32 LF (types 3 / 4) 3-5/8" stud; define member / elevation; if not required: minus both.</t>
@@ -1822,7 +1834,7 @@
     <t xml:space="preserve">RFI-53</t>
   </si>
   <si>
-    <t xml:space="preserve">Light fixtures in the Cafe GWB bands (11'-6" and 9'-0", 1/A-121): fixture count in the bands not taken; 5/A-121 "PROVIDE ADDITIONAL WIRE SUPPORT AT ALL LIGHT FIXTURES". Paso 12 2nd pass (rev8): E-301 Sec. 265119: "THIS CONTRACTOR SHALL PROVIDE AND INSTALL ALL NECESSARY SUPPORT MEDIA FOR ALL LIGHTING FIXTURES ... FIXTURES SHALL NOT BE SUPPORTED FROM ROOF DECK" - overlap with the 5/A-121 fixture wires carried.</t>
+    <t xml:space="preserve">Light fixtures in the Cafe GWB bands (11'-6" and 9'-0", 1/A-121): fixture count in the bands not taken; 5/A-121 "PROVIDE ADDITIONAL WIRE SUPPORT AT ALL LIGHT FIXTURES". Plan check (rev8): E-301 Sec. 265119: "THIS CONTRACTOR SHALL PROVIDE AND INSTALL ALL NECESSARY SUPPORT MEDIA FOR ALL LIGHTING FIXTURES ... FIXTURES SHALL NOT BE SUPPORTED FROM ROOF DECK" - overlap with the 5/A-121 fixture wires carried.</t>
   </si>
   <si>
     <t xml:space="preserve">Each fixture in a band = + 1 hanger x 13.5 / 16.0 ft wire. If the fixture supports are by the electrical contractor (E-301 265119): - 401.0 LF hanger wire (29 hangers).</t>
@@ -1834,7 +1846,7 @@
     <t xml:space="preserve">Fastener counts not printed: 7/A-210 3"x3"x16 ga clip angles (count per header end); cement board screw spacing (manufacturer standard 8" O.C. used); plywood screws per A-410 note 8.D (24" field / 12" perimeter on 4x8 sheets).</t>
   </si>
   <si>
-    <t xml:space="preserve">Carried: clip angles 7/A-210 4 pcs; cement board screws 1686 pcs; plywood screws 2331 pcs - adjust to the estimator yields. Framing screws count the stud pieces of the walls and column wraps (781); the detail members (braces, cross members, posts, bracing) add about + 724 screws. Slab pins at 12" O.C. (estimator criterion); A-410 note 8.F (2 rows at 16" O.C. into concrete) = about + 321 pins. Paso 12 2nd pass (rev8): relief channel to structure carried with 8/A-410 #8 pan head screws (291 pcs) + P.A.F. at cross members (282 pcs); note 8.C X-EDNI (2 rows @ 16" = 720 pcs) is the alternative if the track bears directly on structural steel. Slab pins carried per note 8.F (2 rows @ 16" X-DNI); 9/A-410 alternative 0.177" PAF @ 24" = - 640.61 pcs.</t>
+    <t xml:space="preserve">Carried: clip angles 7/A-210 4 pcs; cement board screws 1686 pcs; plywood screws 2331 pcs - adjust to the estimator yields. Framing screws count the stud pieces of the walls and column wraps (781); the detail members (braces, cross members, bracing) add about + 724 screws. 9/A-410 calls #8 screws stud to track while note 8.A calls #10-16 on 18/16 ga - carried per 8.A. Plan check (rev8): relief channel to structure carried with 8/A-410 #8 pan head screws (291 pcs) + P.A.F. at cross members (282 pcs); note 8.C X-EDNI (2 rows @ 16" = 720 pcs) is the alternative if the track bears directly on structural steel. Slab pins carried per note 8.F (2 rows @ 16" X-DNI); 9/A-410 alternative 0.177" PAF @ 24" = - 640.61 pcs.</t>
   </si>
   <si>
     <t xml:space="preserve">0 questions in total, asked ONE at a time in this order: floor plan (partition types A-Z), then the details the floor plan calls, in order</t>
@@ -2146,7 +2158,7 @@
     <t xml:space="preserve">reglas.py compuerta OK</t>
   </si>
   <si>
-    <t xml:space="preserve">{"canon": "8871f000e4f283aaf53e21edf6ab1d23b08293597a83da947bcd4f1afdb37dfc", "evidencias": "82f4ec13c901d7191f9772989e98854d158340ab19499f6cfbada96ca6cbd21e", "familias_out": "e3b56e640194c143904e80d83c876a670eee27cbf90e467055cb02c7932176be", "reglas": "e6de403e47b5aff83e6ca5064f657f448b59ec1e6bbfaf2c2faf6ce87f8729ce", "version": "v73"}</t>
+    <t xml:space="preserve">{"canon": "10f5767fbe6d10175f7550f9277cd486c29266b3548a6196084574efbcbdf683", "evidencias": "82f4ec13c901d7191f9772989e98854d158340ab19499f6cfbada96ca6cbd21e", "familias_out": "5e80b25c4c58f2a7c1ce346a2e981b61dd297fac8c01d5924de335dd8fefe16b", "reglas": "e6de403e47b5aff83e6ca5064f657f448b59ec1e6bbfaf2c2faf6ce87f8729ce", "version": "v73"}</t>
   </si>
 </sst>
 </file>
@@ -5600,7 +5612,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:J57"/>
+  <dimension ref="A1:J59"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="60"/>
@@ -6092,7 +6104,7 @@
         <v>325</v>
       </c>
       <c r="C17" s="0" t="n">
-        <v>2821.21</v>
+        <v>2689.79</v>
       </c>
       <c r="D17" s="0" t="n">
         <f aca="false">Inputs!$B$5</f>
@@ -6100,18 +6112,18 @@
       </c>
       <c r="E17" s="0" t="n">
         <f aca="false">C17*D17</f>
-        <v>423.1815</v>
+        <v>403.4685</v>
       </c>
       <c r="F17" s="0" t="n">
         <f aca="false">C17+E17</f>
-        <v>3244.3915</v>
+        <v>3093.2585</v>
       </c>
       <c r="G17" s="0" t="s">
         <v>33</v>
       </c>
       <c r="H17" s="0" t="n">
         <f aca="false">ROUNDUP(F17,0)</f>
-        <v>3245</v>
+        <v>3094</v>
       </c>
       <c r="I17" s="0" t="s">
         <v>353</v>
@@ -6455,7 +6467,7 @@
         <v>371</v>
       </c>
       <c r="C28" s="0" t="n">
-        <v>282</v>
+        <v>10088</v>
       </c>
       <c r="D28" s="0" t="n">
         <f aca="false">Inputs!$B$5</f>
@@ -6463,18 +6475,18 @@
       </c>
       <c r="E28" s="0" t="n">
         <f aca="false">C28*D28</f>
-        <v>42.3</v>
+        <v>1513.2</v>
       </c>
       <c r="F28" s="0" t="n">
         <f aca="false">C28+E28</f>
-        <v>324.3</v>
+        <v>11601.2</v>
       </c>
       <c r="G28" s="0" t="s">
         <v>355</v>
       </c>
       <c r="H28" s="0" t="n">
         <f aca="false">ROUNDUP(F28,0)</f>
-        <v>325</v>
+        <v>11602</v>
       </c>
       <c r="I28" s="0" t="s">
         <v>376</v>
@@ -6485,29 +6497,29 @@
         <v>377</v>
       </c>
       <c r="B29" s="0" t="s">
-        <v>358</v>
+        <v>325</v>
       </c>
       <c r="C29" s="0" t="n">
-        <v>50.04</v>
+        <v>131.42</v>
       </c>
       <c r="D29" s="0" t="n">
-        <f aca="false">Inputs!$B$6</f>
-        <v>0.06</v>
+        <f aca="false">Inputs!$B$5</f>
+        <v>0.15</v>
       </c>
       <c r="E29" s="0" t="n">
         <f aca="false">C29*D29</f>
-        <v>3.0024</v>
+        <v>19.713</v>
       </c>
       <c r="F29" s="0" t="n">
         <f aca="false">C29+E29</f>
-        <v>53.0424</v>
+        <v>151.133</v>
       </c>
       <c r="G29" s="0" t="s">
-        <v>359</v>
+        <v>355</v>
       </c>
       <c r="H29" s="0" t="n">
-        <f aca="false">ROUNDUP(F29/Inputs!$B$9,0)</f>
-        <v>2</v>
+        <f aca="false">ROUNDUP(F29,0)</f>
+        <v>152</v>
       </c>
       <c r="I29" s="0" t="s">
         <v>378</v>
@@ -6521,7 +6533,7 @@
         <v>371</v>
       </c>
       <c r="C30" s="0" t="n">
-        <v>2331</v>
+        <v>282</v>
       </c>
       <c r="D30" s="0" t="n">
         <f aca="false">Inputs!$B$5</f>
@@ -6529,18 +6541,18 @@
       </c>
       <c r="E30" s="0" t="n">
         <f aca="false">C30*D30</f>
-        <v>349.65</v>
+        <v>42.3</v>
       </c>
       <c r="F30" s="0" t="n">
         <f aca="false">C30+E30</f>
-        <v>2680.65</v>
+        <v>324.3</v>
       </c>
       <c r="G30" s="0" t="s">
         <v>355</v>
       </c>
       <c r="H30" s="0" t="n">
         <f aca="false">ROUNDUP(F30,0)</f>
-        <v>2681</v>
+        <v>325</v>
       </c>
       <c r="I30" s="0" t="s">
         <v>380</v>
@@ -6551,29 +6563,29 @@
         <v>381</v>
       </c>
       <c r="B31" s="0" t="s">
-        <v>371</v>
+        <v>358</v>
       </c>
       <c r="C31" s="0" t="n">
-        <v>1686</v>
+        <v>50.04</v>
       </c>
       <c r="D31" s="0" t="n">
-        <f aca="false">Inputs!$B$5</f>
-        <v>0.15</v>
+        <f aca="false">Inputs!$B$6</f>
+        <v>0.06</v>
       </c>
       <c r="E31" s="0" t="n">
         <f aca="false">C31*D31</f>
-        <v>252.9</v>
+        <v>3.0024</v>
       </c>
       <c r="F31" s="0" t="n">
         <f aca="false">C31+E31</f>
-        <v>1938.9</v>
+        <v>53.0424</v>
       </c>
       <c r="G31" s="0" t="s">
-        <v>355</v>
+        <v>359</v>
       </c>
       <c r="H31" s="0" t="n">
-        <f aca="false">ROUNDUP(F31,0)</f>
-        <v>1939</v>
+        <f aca="false">ROUNDUP(F31/Inputs!$B$9,0)</f>
+        <v>2</v>
       </c>
       <c r="I31" s="0" t="s">
         <v>382</v>
@@ -6584,10 +6596,10 @@
         <v>383</v>
       </c>
       <c r="B32" s="0" t="s">
-        <v>325</v>
+        <v>371</v>
       </c>
       <c r="C32" s="0" t="n">
-        <v>479.85</v>
+        <v>2331</v>
       </c>
       <c r="D32" s="0" t="n">
         <f aca="false">Inputs!$B$5</f>
@@ -6595,18 +6607,18 @@
       </c>
       <c r="E32" s="0" t="n">
         <f aca="false">C32*D32</f>
-        <v>71.9775</v>
+        <v>349.65</v>
       </c>
       <c r="F32" s="0" t="n">
         <f aca="false">C32+E32</f>
-        <v>551.8275</v>
+        <v>2680.65</v>
       </c>
       <c r="G32" s="0" t="s">
-        <v>326</v>
+        <v>355</v>
       </c>
       <c r="H32" s="0" t="n">
-        <f aca="false">ROUNDUP(F32/Inputs!$B$11,0)</f>
-        <v>56</v>
+        <f aca="false">ROUNDUP(F32,0)</f>
+        <v>2681</v>
       </c>
       <c r="I32" s="0" t="s">
         <v>384</v>
@@ -6617,10 +6629,10 @@
         <v>385</v>
       </c>
       <c r="B33" s="0" t="s">
-        <v>325</v>
+        <v>371</v>
       </c>
       <c r="C33" s="0" t="n">
-        <v>957.03</v>
+        <v>1686</v>
       </c>
       <c r="D33" s="0" t="n">
         <f aca="false">Inputs!$B$5</f>
@@ -6628,65 +6640,65 @@
       </c>
       <c r="E33" s="0" t="n">
         <f aca="false">C33*D33</f>
-        <v>143.5545</v>
+        <v>252.9</v>
       </c>
       <c r="F33" s="0" t="n">
         <f aca="false">C33+E33</f>
-        <v>1100.5845</v>
+        <v>1938.9</v>
       </c>
       <c r="G33" s="0" t="s">
+        <v>355</v>
+      </c>
+      <c r="H33" s="0" t="n">
+        <f aca="false">ROUNDUP(F33,0)</f>
+        <v>1939</v>
+      </c>
+      <c r="I33" s="0" t="s">
         <v>386</v>
-      </c>
-      <c r="H33" s="0" t="n">
-        <f aca="false">ROUNDUP(F33/Inputs!$B$18,0)</f>
-        <v>111</v>
-      </c>
-      <c r="I33" s="0" t="s">
-        <v>387</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="0" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
       <c r="B34" s="0" t="s">
-        <v>358</v>
+        <v>325</v>
       </c>
       <c r="C34" s="0" t="n">
-        <v>739.9</v>
+        <v>479.85</v>
       </c>
       <c r="D34" s="0" t="n">
-        <f aca="false">Inputs!$B$6</f>
-        <v>0.06</v>
+        <f aca="false">Inputs!$B$5</f>
+        <v>0.15</v>
       </c>
       <c r="E34" s="0" t="n">
         <f aca="false">C34*D34</f>
-        <v>44.394</v>
+        <v>71.9775</v>
       </c>
       <c r="F34" s="0" t="n">
         <f aca="false">C34+E34</f>
-        <v>784.294</v>
+        <v>551.8275</v>
       </c>
       <c r="G34" s="0" t="s">
-        <v>359</v>
+        <v>326</v>
       </c>
       <c r="H34" s="0" t="n">
-        <f aca="false">ROUNDUP(F34/Inputs!$B$9,0)</f>
-        <v>17</v>
+        <f aca="false">ROUNDUP(F34/Inputs!$B$11,0)</f>
+        <v>56</v>
       </c>
       <c r="I34" s="0" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="0" t="s">
-        <v>390</v>
+        <v>389</v>
       </c>
       <c r="B35" s="0" t="s">
         <v>325</v>
       </c>
       <c r="C35" s="0" t="n">
-        <v>61.31</v>
+        <v>957.03</v>
       </c>
       <c r="D35" s="0" t="n">
         <f aca="false">Inputs!$B$5</f>
@@ -6694,18 +6706,18 @@
       </c>
       <c r="E35" s="0" t="n">
         <f aca="false">C35*D35</f>
-        <v>9.1965</v>
+        <v>143.5545</v>
       </c>
       <c r="F35" s="0" t="n">
         <f aca="false">C35+E35</f>
-        <v>70.5065</v>
+        <v>1100.5845</v>
       </c>
       <c r="G35" s="0" t="s">
-        <v>336</v>
+        <v>390</v>
       </c>
       <c r="H35" s="0" t="n">
-        <f aca="false">ROUNDUP(F35/Inputs!$B$10,0)</f>
-        <v>4</v>
+        <f aca="false">ROUNDUP(F35/Inputs!$B$18,0)</f>
+        <v>111</v>
       </c>
       <c r="I35" s="0" t="s">
         <v>391</v>
@@ -6716,29 +6728,29 @@
         <v>392</v>
       </c>
       <c r="B36" s="0" t="s">
-        <v>325</v>
+        <v>358</v>
       </c>
       <c r="C36" s="0" t="n">
-        <v>17</v>
+        <v>739.9</v>
       </c>
       <c r="D36" s="0" t="n">
-        <f aca="false">Inputs!$B$5</f>
-        <v>0.15</v>
+        <f aca="false">Inputs!$B$6</f>
+        <v>0.06</v>
       </c>
       <c r="E36" s="0" t="n">
         <f aca="false">C36*D36</f>
-        <v>2.55</v>
+        <v>44.394</v>
       </c>
       <c r="F36" s="0" t="n">
         <f aca="false">C36+E36</f>
-        <v>19.55</v>
+        <v>784.294</v>
       </c>
       <c r="G36" s="0" t="s">
-        <v>355</v>
+        <v>359</v>
       </c>
       <c r="H36" s="0" t="n">
-        <f aca="false">ROUNDUP(F36,0)</f>
-        <v>20</v>
+        <f aca="false">ROUNDUP(F36/Inputs!$B$9,0)</f>
+        <v>17</v>
       </c>
       <c r="I36" s="0" t="s">
         <v>393</v>
@@ -6749,29 +6761,29 @@
         <v>394</v>
       </c>
       <c r="B37" s="0" t="s">
-        <v>358</v>
+        <v>325</v>
       </c>
       <c r="C37" s="0" t="n">
-        <v>1790.51</v>
+        <v>61.31</v>
       </c>
       <c r="D37" s="0" t="n">
-        <f aca="false">Inputs!$B$6</f>
-        <v>0.06</v>
+        <f aca="false">Inputs!$B$5</f>
+        <v>0.15</v>
       </c>
       <c r="E37" s="0" t="n">
         <f aca="false">C37*D37</f>
-        <v>107.4306</v>
+        <v>9.1965</v>
       </c>
       <c r="F37" s="0" t="n">
         <f aca="false">C37+E37</f>
-        <v>1897.9406</v>
+        <v>70.5065</v>
       </c>
       <c r="G37" s="0" t="s">
-        <v>359</v>
+        <v>336</v>
       </c>
       <c r="H37" s="0" t="n">
-        <f aca="false">ROUNDUP(F37/Inputs!$B$9,0)</f>
-        <v>40</v>
+        <f aca="false">ROUNDUP(F37/Inputs!$B$10,0)</f>
+        <v>4</v>
       </c>
       <c r="I37" s="0" t="s">
         <v>395</v>
@@ -6782,29 +6794,29 @@
         <v>396</v>
       </c>
       <c r="B38" s="0" t="s">
-        <v>358</v>
+        <v>325</v>
       </c>
       <c r="C38" s="0" t="n">
-        <v>402.46</v>
+        <v>17</v>
       </c>
       <c r="D38" s="0" t="n">
-        <f aca="false">Inputs!$B$6</f>
-        <v>0.06</v>
+        <f aca="false">Inputs!$B$5</f>
+        <v>0.15</v>
       </c>
       <c r="E38" s="0" t="n">
         <f aca="false">C38*D38</f>
-        <v>24.1476</v>
+        <v>2.55</v>
       </c>
       <c r="F38" s="0" t="n">
         <f aca="false">C38+E38</f>
-        <v>426.6076</v>
+        <v>19.55</v>
       </c>
       <c r="G38" s="0" t="s">
-        <v>359</v>
+        <v>355</v>
       </c>
       <c r="H38" s="0" t="n">
-        <f aca="false">ROUNDUP(F38/Inputs!$B$9,0)</f>
-        <v>9</v>
+        <f aca="false">ROUNDUP(F38,0)</f>
+        <v>20</v>
       </c>
       <c r="I38" s="0" t="s">
         <v>397</v>
@@ -6815,25 +6827,29 @@
         <v>398</v>
       </c>
       <c r="B39" s="0" t="s">
-        <v>371</v>
+        <v>358</v>
       </c>
       <c r="C39" s="0" t="n">
-        <v>109</v>
+        <v>1790.51</v>
       </c>
       <c r="D39" s="0" t="n">
-        <v>0</v>
+        <f aca="false">Inputs!$B$6</f>
+        <v>0.06</v>
       </c>
       <c r="E39" s="0" t="n">
         <f aca="false">C39*D39</f>
-        <v>0</v>
+        <v>107.4306</v>
       </c>
       <c r="F39" s="0" t="n">
         <f aca="false">C39+E39</f>
-        <v>109</v>
+        <v>1897.9406</v>
+      </c>
+      <c r="G39" s="0" t="s">
+        <v>359</v>
       </c>
       <c r="H39" s="0" t="n">
-        <f aca="false">ROUNDUP(F39,0)</f>
-        <v>109</v>
+        <f aca="false">ROUNDUP(F39/Inputs!$B$9,0)</f>
+        <v>40</v>
       </c>
       <c r="I39" s="0" t="s">
         <v>399</v>
@@ -6844,29 +6860,29 @@
         <v>400</v>
       </c>
       <c r="B40" s="0" t="s">
-        <v>325</v>
+        <v>358</v>
       </c>
       <c r="C40" s="0" t="n">
-        <v>10.67</v>
+        <v>402.46</v>
       </c>
       <c r="D40" s="0" t="n">
-        <f aca="false">Inputs!$B$5</f>
-        <v>0.15</v>
+        <f aca="false">Inputs!$B$6</f>
+        <v>0.06</v>
       </c>
       <c r="E40" s="0" t="n">
         <f aca="false">C40*D40</f>
-        <v>1.6005</v>
+        <v>24.1476</v>
       </c>
       <c r="F40" s="0" t="n">
         <f aca="false">C40+E40</f>
-        <v>12.2705</v>
+        <v>426.6076</v>
       </c>
       <c r="G40" s="0" t="s">
-        <v>326</v>
+        <v>359</v>
       </c>
       <c r="H40" s="0" t="n">
-        <f aca="false">ROUNDUP(F40/Inputs!$B$11,0)</f>
-        <v>2</v>
+        <f aca="false">ROUNDUP(F40/Inputs!$B$9,0)</f>
+        <v>9</v>
       </c>
       <c r="I40" s="0" t="s">
         <v>401</v>
@@ -6880,7 +6896,7 @@
         <v>371</v>
       </c>
       <c r="C41" s="0" t="n">
-        <v>0</v>
+        <v>109</v>
       </c>
       <c r="D41" s="0" t="n">
         <v>0</v>
@@ -6891,28 +6907,25 @@
       </c>
       <c r="F41" s="0" t="n">
         <f aca="false">C41+E41</f>
-        <v>0</v>
-      </c>
-      <c r="G41" s="0" t="s">
-        <v>403</v>
+        <v>109</v>
       </c>
       <c r="H41" s="0" t="n">
         <f aca="false">ROUNDUP(F41,0)</f>
-        <v>0</v>
+        <v>109</v>
       </c>
       <c r="I41" s="0" t="s">
-        <v>404</v>
+        <v>403</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="0" t="s">
-        <v>405</v>
+        <v>404</v>
       </c>
       <c r="B42" s="0" t="s">
         <v>325</v>
       </c>
       <c r="C42" s="0" t="n">
-        <v>0</v>
+        <v>10.67</v>
       </c>
       <c r="D42" s="0" t="n">
         <f aca="false">Inputs!$B$5</f>
@@ -6920,36 +6933,35 @@
       </c>
       <c r="E42" s="0" t="n">
         <f aca="false">C42*D42</f>
-        <v>0</v>
+        <v>1.6005</v>
       </c>
       <c r="F42" s="0" t="n">
         <f aca="false">C42+E42</f>
-        <v>0</v>
+        <v>12.2705</v>
       </c>
       <c r="G42" s="0" t="s">
-        <v>336</v>
+        <v>326</v>
       </c>
       <c r="H42" s="0" t="n">
-        <f aca="false">ROUNDUP(F42/Inputs!$B$10,0)</f>
-        <v>0</v>
+        <f aca="false">ROUNDUP(F42/Inputs!$B$11,0)</f>
+        <v>2</v>
       </c>
       <c r="I42" s="0" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="0" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
       <c r="B43" s="0" t="s">
-        <v>325</v>
+        <v>371</v>
       </c>
       <c r="C43" s="0" t="n">
         <v>0</v>
       </c>
       <c r="D43" s="0" t="n">
-        <f aca="false">Inputs!$B$5</f>
-        <v>0.15</v>
+        <v>0</v>
       </c>
       <c r="E43" s="0" t="n">
         <f aca="false">C43*D43</f>
@@ -6960,10 +6972,10 @@
         <v>0</v>
       </c>
       <c r="G43" s="0" t="s">
-        <v>336</v>
+        <v>407</v>
       </c>
       <c r="H43" s="0" t="n">
-        <f aca="false">ROUNDUP(F43/Inputs!$B$10,0)</f>
+        <f aca="false">ROUNDUP(F43,0)</f>
         <v>0</v>
       </c>
       <c r="I43" s="0" t="s">
@@ -6975,14 +6987,14 @@
         <v>409</v>
       </c>
       <c r="B44" s="0" t="s">
-        <v>358</v>
+        <v>325</v>
       </c>
       <c r="C44" s="0" t="n">
         <v>0</v>
       </c>
       <c r="D44" s="0" t="n">
-        <f aca="false">Inputs!$B$6</f>
-        <v>0.06</v>
+        <f aca="false">Inputs!$B$5</f>
+        <v>0.15</v>
       </c>
       <c r="E44" s="0" t="n">
         <f aca="false">C44*D44</f>
@@ -6993,10 +7005,10 @@
         <v>0</v>
       </c>
       <c r="G44" s="0" t="s">
-        <v>359</v>
+        <v>336</v>
       </c>
       <c r="H44" s="0" t="n">
-        <f aca="false">ROUNDUP(F44/Inputs!$B$9,0)</f>
+        <f aca="false">ROUNDUP(F44/Inputs!$B$10,0)</f>
         <v>0</v>
       </c>
       <c r="I44" s="0" t="s">
@@ -7014,8 +7026,8 @@
         <v>0</v>
       </c>
       <c r="D45" s="0" t="n">
-        <f aca="false">Inputs!$B$6</f>
-        <v>0.06</v>
+        <f aca="false">Inputs!$B$5</f>
+        <v>0.15</v>
       </c>
       <c r="E45" s="0" t="n">
         <f aca="false">C45*D45</f>
@@ -7026,10 +7038,10 @@
         <v>0</v>
       </c>
       <c r="G45" s="0" t="s">
-        <v>386</v>
+        <v>336</v>
       </c>
       <c r="H45" s="0" t="n">
-        <f aca="false">ROUNDUP(F45/Inputs!$B$18,0)</f>
+        <f aca="false">ROUNDUP(F45/Inputs!$B$10,0)</f>
         <v>0</v>
       </c>
       <c r="I45" s="0" t="s">
@@ -7041,13 +7053,14 @@
         <v>413</v>
       </c>
       <c r="B46" s="0" t="s">
-        <v>371</v>
+        <v>358</v>
       </c>
       <c r="C46" s="0" t="n">
         <v>0</v>
       </c>
       <c r="D46" s="0" t="n">
-        <v>0</v>
+        <f aca="false">Inputs!$B$6</f>
+        <v>0.06</v>
       </c>
       <c r="E46" s="0" t="n">
         <f aca="false">C46*D46</f>
@@ -7058,10 +7071,10 @@
         <v>0</v>
       </c>
       <c r="G46" s="0" t="s">
-        <v>403</v>
+        <v>359</v>
       </c>
       <c r="H46" s="0" t="n">
-        <f aca="false">ROUNDUP(F46,0)</f>
+        <f aca="false">ROUNDUP(F46/Inputs!$B$9,0)</f>
         <v>0</v>
       </c>
       <c r="I46" s="0" t="s">
@@ -7073,13 +7086,14 @@
         <v>415</v>
       </c>
       <c r="B47" s="0" t="s">
-        <v>371</v>
+        <v>325</v>
       </c>
       <c r="C47" s="0" t="n">
         <v>0</v>
       </c>
       <c r="D47" s="0" t="n">
-        <v>0</v>
+        <f aca="false">Inputs!$B$6</f>
+        <v>0.06</v>
       </c>
       <c r="E47" s="0" t="n">
         <f aca="false">C47*D47</f>
@@ -7090,10 +7104,10 @@
         <v>0</v>
       </c>
       <c r="G47" s="0" t="s">
-        <v>403</v>
+        <v>390</v>
       </c>
       <c r="H47" s="0" t="n">
-        <f aca="false">ROUNDUP(F47,0)</f>
+        <f aca="false">ROUNDUP(F47/Inputs!$B$18,0)</f>
         <v>0</v>
       </c>
       <c r="I47" s="0" t="s">
@@ -7108,7 +7122,7 @@
         <v>371</v>
       </c>
       <c r="C48" s="0" t="n">
-        <v>6402.26</v>
+        <v>0</v>
       </c>
       <c r="D48" s="0" t="n">
         <v>0</v>
@@ -7119,21 +7133,17 @@
       </c>
       <c r="F48" s="0" t="n">
         <f aca="false">C48+E48</f>
-        <v>6402.26</v>
+        <v>0</v>
       </c>
       <c r="G48" s="0" t="s">
-        <v>403</v>
+        <v>407</v>
       </c>
       <c r="H48" s="0" t="n">
         <f aca="false">ROUNDUP(F48,0)</f>
-        <v>6403</v>
+        <v>0</v>
       </c>
       <c r="I48" s="0" t="s">
         <v>418</v>
-      </c>
-      <c r="J48" s="0" t="n">
-        <f aca="false">Inputs!$B$20*5335.22</f>
-        <v>6402.264</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7144,7 +7154,7 @@
         <v>371</v>
       </c>
       <c r="C49" s="0" t="n">
-        <v>1940</v>
+        <v>0</v>
       </c>
       <c r="D49" s="0" t="n">
         <v>0</v>
@@ -7155,21 +7165,17 @@
       </c>
       <c r="F49" s="0" t="n">
         <f aca="false">C49+E49</f>
-        <v>1940</v>
+        <v>0</v>
       </c>
       <c r="G49" s="0" t="s">
-        <v>403</v>
+        <v>407</v>
       </c>
       <c r="H49" s="0" t="n">
         <f aca="false">ROUNDUP(F49,0)</f>
-        <v>1940</v>
+        <v>0</v>
       </c>
       <c r="I49" s="0" t="s">
         <v>420</v>
-      </c>
-      <c r="J49" s="0" t="n">
-        <f aca="false">Inputs!$B$21*485</f>
-        <v>1940</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7180,7 +7186,7 @@
         <v>371</v>
       </c>
       <c r="C50" s="0" t="n">
-        <v>960.91</v>
+        <v>6069.95</v>
       </c>
       <c r="D50" s="0" t="n">
         <v>0</v>
@@ -7191,21 +7197,21 @@
       </c>
       <c r="F50" s="0" t="n">
         <f aca="false">C50+E50</f>
-        <v>960.91</v>
+        <v>6069.95</v>
       </c>
       <c r="G50" s="0" t="s">
-        <v>403</v>
+        <v>407</v>
       </c>
       <c r="H50" s="0" t="n">
         <f aca="false">ROUNDUP(F50,0)</f>
-        <v>961</v>
+        <v>6070</v>
       </c>
       <c r="I50" s="0" t="s">
         <v>422</v>
       </c>
       <c r="J50" s="0" t="n">
-        <f aca="false">640.61/Inputs!$B$22</f>
-        <v>960.91451954274</v>
+        <f aca="false">Inputs!$B$20*5058.29</f>
+        <v>6069.948</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7216,7 +7222,7 @@
         <v>371</v>
       </c>
       <c r="C51" s="0" t="n">
-        <v>0</v>
+        <v>1940</v>
       </c>
       <c r="D51" s="0" t="n">
         <v>0</v>
@@ -7227,21 +7233,21 @@
       </c>
       <c r="F51" s="0" t="n">
         <f aca="false">C51+E51</f>
-        <v>0</v>
+        <v>1940</v>
       </c>
       <c r="G51" s="0" t="s">
-        <v>403</v>
+        <v>407</v>
       </c>
       <c r="H51" s="0" t="n">
         <f aca="false">ROUNDUP(F51,0)</f>
-        <v>0</v>
+        <v>1940</v>
       </c>
       <c r="I51" s="0" t="s">
         <v>424</v>
       </c>
       <c r="J51" s="0" t="n">
-        <f aca="false">0*Inputs!$B$25</f>
-        <v>0</v>
+        <f aca="false">Inputs!$B$21*485</f>
+        <v>1940</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7249,10 +7255,10 @@
         <v>425</v>
       </c>
       <c r="B52" s="0" t="s">
-        <v>426</v>
+        <v>371</v>
       </c>
       <c r="C52" s="0" t="n">
-        <v>1166.54</v>
+        <v>960.91</v>
       </c>
       <c r="D52" s="0" t="n">
         <v>0</v>
@@ -7263,32 +7269,32 @@
       </c>
       <c r="F52" s="0" t="n">
         <f aca="false">C52+E52</f>
-        <v>1166.54</v>
+        <v>960.91</v>
       </c>
       <c r="G52" s="0" t="s">
-        <v>427</v>
+        <v>407</v>
       </c>
       <c r="H52" s="0" t="n">
         <f aca="false">ROUNDUP(F52,0)</f>
-        <v>1167</v>
+        <v>961</v>
       </c>
       <c r="I52" s="0" t="s">
-        <v>428</v>
+        <v>426</v>
       </c>
       <c r="J52" s="0" t="n">
-        <f aca="false">Inputs!$B$23*16201.9</f>
-        <v>1166.5368</v>
+        <f aca="false">640.61/Inputs!$B$22</f>
+        <v>960.91451954274</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="0" t="s">
-        <v>429</v>
+        <v>427</v>
       </c>
       <c r="B53" s="0" t="s">
-        <v>325</v>
+        <v>371</v>
       </c>
       <c r="C53" s="0" t="n">
-        <v>5994.7</v>
+        <v>0</v>
       </c>
       <c r="D53" s="0" t="n">
         <v>0</v>
@@ -7299,36 +7305,35 @@
       </c>
       <c r="F53" s="0" t="n">
         <f aca="false">C53+E53</f>
-        <v>5994.7</v>
+        <v>0</v>
       </c>
       <c r="G53" s="0" t="s">
-        <v>325</v>
+        <v>407</v>
       </c>
       <c r="H53" s="0" t="n">
         <f aca="false">ROUNDUP(F53,0)</f>
-        <v>5995</v>
+        <v>0</v>
       </c>
       <c r="I53" s="0" t="s">
-        <v>430</v>
+        <v>428</v>
       </c>
       <c r="J53" s="0" t="n">
-        <f aca="false">Inputs!$B$24*16201.9</f>
-        <v>5994.703</v>
+        <f aca="false">0*Inputs!$B$25</f>
+        <v>0</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="0" t="s">
-        <v>431</v>
+        <v>429</v>
       </c>
       <c r="B54" s="0" t="s">
-        <v>358</v>
+        <v>430</v>
       </c>
       <c r="C54" s="0" t="n">
+        <v>1166.54</v>
+      </c>
+      <c r="D54" s="0" t="n">
         <v>0</v>
-      </c>
-      <c r="D54" s="0" t="n">
-        <f aca="false">Inputs!$B$6</f>
-        <v>0.06</v>
       </c>
       <c r="E54" s="0" t="n">
         <f aca="false">C54*D54</f>
@@ -7336,17 +7341,21 @@
       </c>
       <c r="F54" s="0" t="n">
         <f aca="false">C54+E54</f>
-        <v>0</v>
+        <v>1166.54</v>
       </c>
       <c r="G54" s="0" t="s">
-        <v>358</v>
+        <v>431</v>
       </c>
       <c r="H54" s="0" t="n">
         <f aca="false">ROUNDUP(F54,0)</f>
-        <v>0</v>
+        <v>1167</v>
       </c>
       <c r="I54" s="0" t="s">
         <v>432</v>
+      </c>
+      <c r="J54" s="0" t="n">
+        <f aca="false">Inputs!$B$23*16201.9</f>
+        <v>1166.5368</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7354,10 +7363,10 @@
         <v>433</v>
       </c>
       <c r="B55" s="0" t="s">
-        <v>371</v>
+        <v>325</v>
       </c>
       <c r="C55" s="0" t="n">
-        <v>0</v>
+        <v>5994.7</v>
       </c>
       <c r="D55" s="0" t="n">
         <v>0</v>
@@ -7368,17 +7377,21 @@
       </c>
       <c r="F55" s="0" t="n">
         <f aca="false">C55+E55</f>
-        <v>0</v>
+        <v>5994.7</v>
       </c>
       <c r="G55" s="0" t="s">
-        <v>403</v>
+        <v>325</v>
       </c>
       <c r="H55" s="0" t="n">
         <f aca="false">ROUNDUP(F55,0)</f>
-        <v>0</v>
+        <v>5995</v>
       </c>
       <c r="I55" s="0" t="s">
         <v>434</v>
+      </c>
+      <c r="J55" s="0" t="n">
+        <f aca="false">Inputs!$B$24*16201.9</f>
+        <v>5994.703</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7386,13 +7399,14 @@
         <v>435</v>
       </c>
       <c r="B56" s="0" t="s">
-        <v>371</v>
+        <v>358</v>
       </c>
       <c r="C56" s="0" t="n">
-        <v>1776</v>
+        <v>0</v>
       </c>
       <c r="D56" s="0" t="n">
-        <v>0</v>
+        <f aca="false">Inputs!$B$6</f>
+        <v>0.06</v>
       </c>
       <c r="E56" s="0" t="n">
         <f aca="false">C56*D56</f>
@@ -7400,14 +7414,14 @@
       </c>
       <c r="F56" s="0" t="n">
         <f aca="false">C56+E56</f>
-        <v>1776</v>
+        <v>0</v>
       </c>
       <c r="G56" s="0" t="s">
-        <v>403</v>
+        <v>358</v>
       </c>
       <c r="H56" s="0" t="n">
         <f aca="false">ROUNDUP(F56,0)</f>
-        <v>1776</v>
+        <v>0</v>
       </c>
       <c r="I56" s="0" t="s">
         <v>436</v>
@@ -7421,7 +7435,7 @@
         <v>371</v>
       </c>
       <c r="C57" s="0" t="n">
-        <v>13039.99</v>
+        <v>0</v>
       </c>
       <c r="D57" s="0" t="n">
         <v>0</v>
@@ -7432,17 +7446,81 @@
       </c>
       <c r="F57" s="0" t="n">
         <f aca="false">C57+E57</f>
-        <v>13039.99</v>
+        <v>0</v>
       </c>
       <c r="G57" s="0" t="s">
-        <v>403</v>
+        <v>407</v>
       </c>
       <c r="H57" s="0" t="n">
         <f aca="false">ROUNDUP(F57,0)</f>
-        <v>13040</v>
+        <v>0</v>
       </c>
       <c r="I57" s="0" t="s">
         <v>438</v>
+      </c>
+    </row>
+    <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A58" s="0" t="s">
+        <v>439</v>
+      </c>
+      <c r="B58" s="0" t="s">
+        <v>371</v>
+      </c>
+      <c r="C58" s="0" t="n">
+        <v>1776</v>
+      </c>
+      <c r="D58" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="E58" s="0" t="n">
+        <f aca="false">C58*D58</f>
+        <v>0</v>
+      </c>
+      <c r="F58" s="0" t="n">
+        <f aca="false">C58+E58</f>
+        <v>1776</v>
+      </c>
+      <c r="G58" s="0" t="s">
+        <v>407</v>
+      </c>
+      <c r="H58" s="0" t="n">
+        <f aca="false">ROUNDUP(F58,0)</f>
+        <v>1776</v>
+      </c>
+      <c r="I58" s="0" t="s">
+        <v>440</v>
+      </c>
+    </row>
+    <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A59" s="0" t="s">
+        <v>441</v>
+      </c>
+      <c r="B59" s="0" t="s">
+        <v>371</v>
+      </c>
+      <c r="C59" s="0" t="n">
+        <v>13372.31</v>
+      </c>
+      <c r="D59" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="E59" s="0" t="n">
+        <f aca="false">C59*D59</f>
+        <v>0</v>
+      </c>
+      <c r="F59" s="0" t="n">
+        <f aca="false">C59+E59</f>
+        <v>13372.31</v>
+      </c>
+      <c r="G59" s="0" t="s">
+        <v>407</v>
+      </c>
+      <c r="H59" s="0" t="n">
+        <f aca="false">ROUNDUP(F59,0)</f>
+        <v>13373</v>
+      </c>
+      <c r="I59" s="0" t="s">
+        <v>442</v>
       </c>
     </row>
   </sheetData>
@@ -7470,618 +7548,618 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>439</v>
+        <v>443</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>440</v>
+        <v>444</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>441</v>
+        <v>445</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="0" t="s">
-        <v>442</v>
+        <v>446</v>
       </c>
       <c r="B2" s="0" t="s">
-        <v>443</v>
+        <v>447</v>
       </c>
       <c r="C2" s="0" t="s">
-        <v>444</v>
+        <v>448</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="0" t="s">
-        <v>445</v>
+        <v>449</v>
       </c>
       <c r="B3" s="0" t="s">
-        <v>446</v>
+        <v>450</v>
       </c>
       <c r="C3" s="0" t="s">
-        <v>447</v>
+        <v>451</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="0" t="s">
-        <v>448</v>
+        <v>452</v>
       </c>
       <c r="B4" s="0" t="s">
-        <v>449</v>
+        <v>453</v>
       </c>
       <c r="C4" s="0" t="s">
-        <v>450</v>
+        <v>454</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="0" t="s">
-        <v>451</v>
+        <v>455</v>
       </c>
       <c r="B5" s="0" t="s">
-        <v>452</v>
+        <v>456</v>
       </c>
       <c r="C5" s="0" t="s">
-        <v>453</v>
+        <v>457</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="0" t="s">
-        <v>454</v>
+        <v>458</v>
       </c>
       <c r="B6" s="0" t="s">
-        <v>455</v>
+        <v>459</v>
       </c>
       <c r="C6" s="0" t="s">
-        <v>456</v>
+        <v>460</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="0" t="s">
-        <v>457</v>
+        <v>461</v>
       </c>
       <c r="B7" s="0" t="s">
-        <v>458</v>
+        <v>462</v>
       </c>
       <c r="C7" s="0" t="s">
-        <v>459</v>
+        <v>463</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="0" t="s">
-        <v>460</v>
+        <v>464</v>
       </c>
       <c r="B8" s="0" t="s">
-        <v>461</v>
+        <v>465</v>
       </c>
       <c r="C8" s="0" t="s">
-        <v>462</v>
+        <v>466</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="0" t="s">
-        <v>463</v>
+        <v>467</v>
       </c>
       <c r="B9" s="0" t="s">
-        <v>464</v>
+        <v>468</v>
       </c>
       <c r="C9" s="0" t="s">
-        <v>465</v>
+        <v>469</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="0" t="s">
-        <v>466</v>
+        <v>470</v>
       </c>
       <c r="B10" s="0" t="s">
-        <v>467</v>
+        <v>471</v>
       </c>
       <c r="C10" s="0" t="s">
-        <v>453</v>
+        <v>457</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="0" t="s">
-        <v>468</v>
+        <v>472</v>
       </c>
       <c r="B11" s="0" t="s">
-        <v>469</v>
+        <v>473</v>
       </c>
       <c r="C11" s="0" t="s">
-        <v>470</v>
+        <v>474</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="0" t="s">
-        <v>471</v>
+        <v>475</v>
       </c>
       <c r="B12" s="0" t="s">
-        <v>472</v>
+        <v>476</v>
       </c>
       <c r="C12" s="0" t="s">
-        <v>473</v>
+        <v>477</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="0" t="s">
-        <v>474</v>
+        <v>478</v>
       </c>
       <c r="B13" s="0" t="s">
-        <v>475</v>
+        <v>479</v>
       </c>
       <c r="C13" s="0" t="s">
-        <v>453</v>
+        <v>457</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="0" t="s">
-        <v>476</v>
+        <v>480</v>
       </c>
       <c r="B14" s="0" t="s">
-        <v>477</v>
+        <v>481</v>
       </c>
       <c r="C14" s="0" t="s">
-        <v>478</v>
+        <v>482</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="0" t="s">
-        <v>479</v>
+        <v>483</v>
       </c>
       <c r="B15" s="0" t="s">
-        <v>480</v>
+        <v>484</v>
       </c>
       <c r="C15" s="0" t="s">
-        <v>481</v>
+        <v>485</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="0" t="s">
-        <v>482</v>
+        <v>486</v>
       </c>
       <c r="B16" s="0" t="s">
-        <v>483</v>
+        <v>487</v>
       </c>
       <c r="C16" s="0" t="s">
-        <v>484</v>
+        <v>488</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="0" t="s">
-        <v>485</v>
+        <v>489</v>
       </c>
       <c r="B17" s="0" t="s">
-        <v>486</v>
+        <v>490</v>
       </c>
       <c r="C17" s="0" t="s">
-        <v>487</v>
+        <v>491</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="0" t="s">
-        <v>488</v>
+        <v>492</v>
       </c>
       <c r="B18" s="0" t="s">
-        <v>489</v>
+        <v>493</v>
       </c>
       <c r="C18" s="0" t="s">
-        <v>490</v>
+        <v>494</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="0" t="s">
-        <v>491</v>
+        <v>495</v>
       </c>
       <c r="B19" s="0" t="s">
-        <v>492</v>
+        <v>496</v>
       </c>
       <c r="C19" s="0" t="s">
-        <v>493</v>
+        <v>497</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="0" t="s">
-        <v>494</v>
+        <v>498</v>
       </c>
       <c r="B20" s="0" t="s">
-        <v>495</v>
+        <v>499</v>
       </c>
       <c r="C20" s="0" t="s">
-        <v>496</v>
+        <v>500</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="0" t="s">
-        <v>497</v>
+        <v>501</v>
       </c>
       <c r="B21" s="0" t="s">
-        <v>498</v>
+        <v>502</v>
       </c>
       <c r="C21" s="0" t="s">
-        <v>499</v>
+        <v>503</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="0" t="s">
-        <v>500</v>
+        <v>504</v>
       </c>
       <c r="B22" s="0" t="s">
-        <v>501</v>
+        <v>505</v>
       </c>
       <c r="C22" s="0" t="s">
-        <v>453</v>
+        <v>457</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="0" t="s">
-        <v>502</v>
+        <v>506</v>
       </c>
       <c r="B23" s="0" t="s">
-        <v>503</v>
+        <v>507</v>
       </c>
       <c r="C23" s="0" t="s">
-        <v>504</v>
+        <v>508</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="0" t="s">
-        <v>505</v>
+        <v>509</v>
       </c>
       <c r="B24" s="0" t="s">
-        <v>506</v>
+        <v>510</v>
       </c>
       <c r="C24" s="0" t="s">
-        <v>507</v>
+        <v>511</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="0" t="s">
-        <v>508</v>
+        <v>512</v>
       </c>
       <c r="B25" s="0" t="s">
-        <v>509</v>
+        <v>513</v>
       </c>
       <c r="C25" s="0" t="s">
-        <v>510</v>
+        <v>514</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="0" t="s">
-        <v>511</v>
+        <v>515</v>
       </c>
       <c r="B26" s="0" t="s">
-        <v>512</v>
+        <v>516</v>
       </c>
       <c r="C26" s="0" t="s">
-        <v>513</v>
+        <v>517</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="0" t="s">
-        <v>514</v>
+        <v>518</v>
       </c>
       <c r="B27" s="0" t="s">
-        <v>515</v>
+        <v>519</v>
       </c>
       <c r="C27" s="0" t="s">
-        <v>516</v>
+        <v>520</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="0" t="s">
-        <v>517</v>
+        <v>521</v>
       </c>
       <c r="B28" s="0" t="s">
-        <v>518</v>
+        <v>522</v>
       </c>
       <c r="C28" s="0" t="s">
-        <v>519</v>
+        <v>523</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="0" t="s">
-        <v>520</v>
+        <v>524</v>
       </c>
       <c r="B29" s="0" t="s">
-        <v>521</v>
+        <v>525</v>
       </c>
       <c r="C29" s="0" t="s">
-        <v>453</v>
+        <v>457</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="0" t="s">
-        <v>522</v>
+        <v>526</v>
       </c>
       <c r="B30" s="0" t="s">
-        <v>523</v>
+        <v>527</v>
       </c>
       <c r="C30" s="0" t="s">
-        <v>524</v>
+        <v>528</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="0" t="s">
-        <v>525</v>
+        <v>529</v>
       </c>
       <c r="B31" s="0" t="s">
-        <v>526</v>
+        <v>530</v>
       </c>
       <c r="C31" s="0" t="s">
-        <v>527</v>
+        <v>531</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="0" t="s">
-        <v>528</v>
+        <v>532</v>
       </c>
       <c r="B32" s="0" t="s">
-        <v>529</v>
+        <v>533</v>
       </c>
       <c r="C32" s="0" t="s">
-        <v>530</v>
+        <v>534</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="0" t="s">
-        <v>531</v>
+        <v>535</v>
       </c>
       <c r="B33" s="0" t="s">
-        <v>532</v>
+        <v>536</v>
       </c>
       <c r="C33" s="0" t="s">
-        <v>533</v>
+        <v>537</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="0" t="s">
-        <v>534</v>
+        <v>538</v>
       </c>
       <c r="B34" s="0" t="s">
-        <v>535</v>
+        <v>539</v>
       </c>
       <c r="C34" s="0" t="s">
-        <v>536</v>
+        <v>540</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="0" t="s">
-        <v>537</v>
+        <v>541</v>
       </c>
       <c r="B35" s="0" t="s">
-        <v>538</v>
+        <v>542</v>
       </c>
       <c r="C35" s="0" t="s">
-        <v>539</v>
+        <v>543</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="0" t="s">
-        <v>540</v>
+        <v>544</v>
       </c>
       <c r="B36" s="0" t="s">
-        <v>541</v>
+        <v>545</v>
       </c>
       <c r="C36" s="0" t="s">
-        <v>542</v>
+        <v>546</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="0" t="s">
-        <v>543</v>
+        <v>547</v>
       </c>
       <c r="B37" s="0" t="s">
-        <v>544</v>
+        <v>548</v>
       </c>
       <c r="C37" s="0" t="s">
-        <v>545</v>
+        <v>549</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="0" t="s">
-        <v>546</v>
+        <v>550</v>
       </c>
       <c r="B38" s="0" t="s">
-        <v>547</v>
+        <v>551</v>
       </c>
       <c r="C38" s="0" t="s">
-        <v>548</v>
+        <v>552</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="0" t="s">
-        <v>549</v>
+        <v>553</v>
       </c>
       <c r="B39" s="0" t="s">
-        <v>550</v>
+        <v>554</v>
       </c>
       <c r="C39" s="0" t="s">
-        <v>551</v>
+        <v>555</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="0" t="s">
-        <v>552</v>
+        <v>556</v>
       </c>
       <c r="B40" s="0" t="s">
-        <v>553</v>
+        <v>557</v>
       </c>
       <c r="C40" s="0" t="s">
-        <v>554</v>
+        <v>558</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="0" t="s">
-        <v>555</v>
+        <v>559</v>
       </c>
       <c r="B41" s="0" t="s">
-        <v>556</v>
+        <v>560</v>
       </c>
       <c r="C41" s="0" t="s">
-        <v>557</v>
+        <v>561</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="0" t="s">
-        <v>558</v>
+        <v>562</v>
       </c>
       <c r="B42" s="0" t="s">
-        <v>559</v>
+        <v>563</v>
       </c>
       <c r="C42" s="0" t="s">
-        <v>560</v>
+        <v>564</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="0" t="s">
-        <v>561</v>
+        <v>565</v>
       </c>
       <c r="B43" s="0" t="s">
-        <v>562</v>
+        <v>566</v>
       </c>
       <c r="C43" s="0" t="s">
-        <v>563</v>
+        <v>567</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="0" t="s">
-        <v>564</v>
+        <v>568</v>
       </c>
       <c r="B44" s="0" t="s">
-        <v>565</v>
+        <v>569</v>
       </c>
       <c r="C44" s="0" t="s">
-        <v>566</v>
+        <v>570</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="0" t="s">
-        <v>567</v>
+        <v>571</v>
       </c>
       <c r="B45" s="0" t="s">
-        <v>568</v>
+        <v>572</v>
       </c>
       <c r="C45" s="0" t="s">
-        <v>569</v>
+        <v>573</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="0" t="s">
-        <v>570</v>
+        <v>574</v>
       </c>
       <c r="B46" s="0" t="s">
-        <v>571</v>
+        <v>575</v>
       </c>
       <c r="C46" s="0" t="s">
-        <v>572</v>
+        <v>576</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="0" t="s">
-        <v>573</v>
+        <v>577</v>
       </c>
       <c r="B47" s="0" t="s">
-        <v>574</v>
+        <v>578</v>
       </c>
       <c r="C47" s="0" t="s">
-        <v>575</v>
+        <v>579</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="0" t="s">
-        <v>576</v>
+        <v>580</v>
       </c>
       <c r="B48" s="0" t="s">
-        <v>577</v>
+        <v>581</v>
       </c>
       <c r="C48" s="0" t="s">
-        <v>578</v>
+        <v>582</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="0" t="s">
-        <v>579</v>
+        <v>583</v>
       </c>
       <c r="B49" s="0" t="s">
-        <v>580</v>
+        <v>584</v>
       </c>
       <c r="C49" s="0" t="s">
-        <v>581</v>
+        <v>585</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="0" t="s">
-        <v>582</v>
+        <v>586</v>
       </c>
       <c r="B50" s="0" t="s">
-        <v>583</v>
+        <v>587</v>
       </c>
       <c r="C50" s="0" t="s">
-        <v>584</v>
+        <v>588</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="0" t="s">
-        <v>585</v>
+        <v>589</v>
       </c>
       <c r="B51" s="0" t="s">
-        <v>586</v>
+        <v>590</v>
       </c>
       <c r="C51" s="0" t="s">
-        <v>587</v>
+        <v>591</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="0" t="s">
-        <v>588</v>
+        <v>592</v>
       </c>
       <c r="B52" s="0" t="s">
-        <v>589</v>
+        <v>593</v>
       </c>
       <c r="C52" s="0" t="s">
-        <v>590</v>
+        <v>594</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="0" t="s">
-        <v>591</v>
+        <v>595</v>
       </c>
       <c r="B53" s="0" t="s">
-        <v>592</v>
+        <v>596</v>
       </c>
       <c r="C53" s="0" t="s">
-        <v>593</v>
+        <v>597</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="0" t="s">
-        <v>594</v>
+        <v>598</v>
       </c>
       <c r="B54" s="0" t="s">
-        <v>595</v>
+        <v>599</v>
       </c>
       <c r="C54" s="0" t="s">
-        <v>596</v>
+        <v>600</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="0" t="s">
-        <v>597</v>
+        <v>601</v>
       </c>
       <c r="B55" s="0" t="s">
-        <v>598</v>
+        <v>602</v>
       </c>
       <c r="C55" s="0" t="s">
-        <v>599</v>
+        <v>603</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="0" t="s">
-        <v>600</v>
+        <v>604</v>
       </c>
       <c r="B56" s="0" t="s">
-        <v>601</v>
+        <v>605</v>
       </c>
       <c r="C56" s="0" t="s">
-        <v>602</v>
+        <v>606</v>
       </c>
     </row>
   </sheetData>
@@ -8113,27 +8191,27 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="0" t="s">
-        <v>603</v>
+        <v>607</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="0" t="s">
-        <v>604</v>
+        <v>608</v>
       </c>
       <c r="B2" s="0" t="s">
-        <v>605</v>
+        <v>609</v>
       </c>
       <c r="C2" s="0" t="s">
-        <v>606</v>
+        <v>610</v>
       </c>
       <c r="D2" s="0" t="s">
-        <v>607</v>
+        <v>611</v>
       </c>
       <c r="E2" s="0" t="s">
-        <v>608</v>
+        <v>612</v>
       </c>
       <c r="F2" s="0" t="s">
-        <v>609</v>
+        <v>613</v>
       </c>
     </row>
   </sheetData>
@@ -8163,436 +8241,436 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="0" t="s">
-        <v>610</v>
+        <v>614</v>
       </c>
       <c r="B1" s="0" t="s">
-        <v>611</v>
+        <v>615</v>
       </c>
       <c r="C1" s="0" t="s">
         <v>59</v>
       </c>
       <c r="D1" s="0" t="s">
-        <v>612</v>
+        <v>616</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="0" t="s">
-        <v>613</v>
+        <v>617</v>
       </c>
       <c r="B2" s="0" t="s">
-        <v>614</v>
+        <v>618</v>
       </c>
       <c r="C2" s="0" t="s">
-        <v>615</v>
+        <v>619</v>
       </c>
       <c r="D2" s="0" t="s">
-        <v>616</v>
+        <v>620</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="0" t="s">
-        <v>617</v>
+        <v>621</v>
       </c>
       <c r="B3" s="0" t="s">
-        <v>618</v>
+        <v>622</v>
       </c>
       <c r="C3" s="0" t="s">
-        <v>619</v>
+        <v>623</v>
       </c>
       <c r="D3" s="0" t="s">
-        <v>620</v>
+        <v>624</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="0" t="s">
-        <v>621</v>
+        <v>625</v>
       </c>
       <c r="B4" s="0" t="s">
-        <v>622</v>
+        <v>626</v>
       </c>
       <c r="C4" s="0" t="s">
-        <v>619</v>
+        <v>623</v>
       </c>
       <c r="D4" s="0" t="s">
-        <v>623</v>
+        <v>627</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="0" t="s">
-        <v>624</v>
+        <v>628</v>
       </c>
       <c r="B5" s="0" t="s">
-        <v>625</v>
+        <v>629</v>
       </c>
       <c r="C5" s="0" t="s">
-        <v>615</v>
+        <v>619</v>
       </c>
       <c r="D5" s="0" t="s">
-        <v>626</v>
+        <v>630</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="0" t="s">
-        <v>627</v>
+        <v>631</v>
       </c>
       <c r="B6" s="0" t="s">
-        <v>628</v>
+        <v>632</v>
       </c>
       <c r="C6" s="0" t="s">
-        <v>439</v>
+        <v>443</v>
       </c>
       <c r="D6" s="0" t="s">
-        <v>629</v>
+        <v>633</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="0" t="s">
-        <v>630</v>
+        <v>634</v>
       </c>
       <c r="B7" s="0" t="s">
-        <v>631</v>
+        <v>635</v>
       </c>
       <c r="C7" s="0" t="s">
-        <v>615</v>
+        <v>619</v>
       </c>
       <c r="D7" s="0" t="s">
-        <v>632</v>
+        <v>636</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="0" t="s">
-        <v>633</v>
+        <v>637</v>
       </c>
       <c r="B8" s="0" t="s">
-        <v>634</v>
+        <v>638</v>
       </c>
       <c r="C8" s="0" t="s">
-        <v>615</v>
+        <v>619</v>
       </c>
       <c r="D8" s="0" t="s">
-        <v>635</v>
+        <v>639</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="0" t="s">
-        <v>636</v>
+        <v>640</v>
       </c>
       <c r="B9" s="0" t="s">
-        <v>637</v>
+        <v>641</v>
       </c>
       <c r="C9" s="0" t="s">
-        <v>615</v>
+        <v>619</v>
       </c>
       <c r="D9" s="0" t="s">
-        <v>638</v>
+        <v>642</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="0" t="s">
-        <v>639</v>
+        <v>643</v>
       </c>
       <c r="B10" s="0" t="s">
-        <v>640</v>
+        <v>644</v>
       </c>
       <c r="C10" s="0" t="s">
-        <v>619</v>
+        <v>623</v>
       </c>
       <c r="D10" s="0" t="s">
-        <v>641</v>
+        <v>645</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="0" t="s">
-        <v>642</v>
+        <v>646</v>
       </c>
       <c r="B11" s="0" t="s">
-        <v>643</v>
+        <v>647</v>
       </c>
       <c r="C11" s="0" t="s">
-        <v>615</v>
+        <v>619</v>
       </c>
       <c r="D11" s="0" t="s">
-        <v>644</v>
+        <v>648</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="0" t="s">
-        <v>645</v>
+        <v>649</v>
       </c>
       <c r="B12" s="0" t="s">
-        <v>646</v>
+        <v>650</v>
       </c>
       <c r="C12" s="0" t="s">
-        <v>615</v>
+        <v>619</v>
       </c>
       <c r="D12" s="0" t="s">
-        <v>647</v>
+        <v>651</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="0" t="s">
-        <v>648</v>
+        <v>652</v>
       </c>
       <c r="B13" s="0" t="s">
-        <v>649</v>
+        <v>653</v>
       </c>
       <c r="C13" s="0" t="s">
-        <v>615</v>
+        <v>619</v>
       </c>
       <c r="D13" s="0" t="s">
-        <v>650</v>
+        <v>654</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="0" t="s">
-        <v>651</v>
+        <v>655</v>
       </c>
       <c r="B14" s="0" t="s">
-        <v>652</v>
+        <v>656</v>
       </c>
       <c r="C14" s="0" t="s">
-        <v>615</v>
+        <v>619</v>
       </c>
       <c r="D14" s="0" t="s">
-        <v>653</v>
+        <v>657</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="0" t="s">
-        <v>654</v>
+        <v>658</v>
       </c>
       <c r="B15" s="0" t="s">
-        <v>655</v>
+        <v>659</v>
       </c>
       <c r="C15" s="0" t="s">
-        <v>619</v>
+        <v>623</v>
       </c>
       <c r="D15" s="0" t="s">
-        <v>656</v>
+        <v>660</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="0" t="s">
-        <v>657</v>
+        <v>661</v>
       </c>
       <c r="B16" s="0" t="s">
-        <v>658</v>
+        <v>662</v>
       </c>
       <c r="C16" s="0" t="s">
-        <v>615</v>
+        <v>619</v>
       </c>
       <c r="D16" s="0" t="s">
-        <v>659</v>
+        <v>663</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="0" t="s">
-        <v>660</v>
+        <v>664</v>
       </c>
       <c r="B17" s="0" t="s">
-        <v>661</v>
+        <v>665</v>
       </c>
       <c r="C17" s="0" t="s">
-        <v>615</v>
+        <v>619</v>
       </c>
       <c r="D17" s="0" t="s">
-        <v>662</v>
+        <v>666</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="0" t="s">
-        <v>663</v>
+        <v>667</v>
       </c>
       <c r="B18" s="0" t="s">
-        <v>664</v>
+        <v>668</v>
       </c>
       <c r="C18" s="0" t="s">
-        <v>439</v>
+        <v>443</v>
       </c>
       <c r="D18" s="0" t="s">
-        <v>665</v>
+        <v>669</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="0" t="s">
-        <v>666</v>
+        <v>670</v>
       </c>
       <c r="B19" s="0" t="s">
-        <v>667</v>
+        <v>671</v>
       </c>
       <c r="C19" s="0" t="s">
-        <v>615</v>
+        <v>619</v>
       </c>
       <c r="D19" s="0" t="s">
-        <v>668</v>
+        <v>672</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="0" t="s">
-        <v>669</v>
+        <v>673</v>
       </c>
       <c r="B20" s="0" t="s">
-        <v>670</v>
+        <v>674</v>
       </c>
       <c r="C20" s="0" t="s">
-        <v>619</v>
+        <v>623</v>
       </c>
       <c r="D20" s="0" t="s">
-        <v>671</v>
+        <v>675</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="0" t="s">
-        <v>672</v>
+        <v>676</v>
       </c>
       <c r="B21" s="0" t="s">
-        <v>673</v>
+        <v>677</v>
       </c>
       <c r="C21" s="0" t="s">
-        <v>615</v>
+        <v>619</v>
       </c>
       <c r="D21" s="0" t="s">
-        <v>674</v>
+        <v>678</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="0" t="s">
-        <v>675</v>
+        <v>679</v>
       </c>
       <c r="B22" s="0" t="s">
-        <v>676</v>
+        <v>680</v>
       </c>
       <c r="C22" s="0" t="s">
-        <v>619</v>
+        <v>623</v>
       </c>
       <c r="D22" s="0" t="s">
-        <v>677</v>
+        <v>681</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="0" t="s">
-        <v>678</v>
+        <v>682</v>
       </c>
       <c r="B23" s="0" t="s">
-        <v>679</v>
+        <v>683</v>
       </c>
       <c r="C23" s="0" t="s">
-        <v>619</v>
+        <v>623</v>
       </c>
       <c r="D23" s="0" t="s">
-        <v>680</v>
+        <v>684</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="0" t="s">
-        <v>681</v>
+        <v>685</v>
       </c>
       <c r="B24" s="0" t="s">
-        <v>682</v>
+        <v>686</v>
       </c>
       <c r="C24" s="0" t="s">
-        <v>619</v>
+        <v>623</v>
       </c>
       <c r="D24" s="0" t="s">
-        <v>683</v>
+        <v>687</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="0" t="s">
-        <v>684</v>
+        <v>688</v>
       </c>
       <c r="B25" s="0" t="s">
-        <v>685</v>
+        <v>689</v>
       </c>
       <c r="C25" s="0" t="s">
-        <v>615</v>
+        <v>619</v>
       </c>
       <c r="D25" s="0" t="s">
-        <v>686</v>
+        <v>690</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="0" t="s">
-        <v>687</v>
+        <v>691</v>
       </c>
       <c r="B26" s="0" t="s">
-        <v>688</v>
+        <v>692</v>
       </c>
       <c r="C26" s="0" t="s">
-        <v>619</v>
+        <v>623</v>
       </c>
       <c r="D26" s="0" t="s">
-        <v>689</v>
+        <v>693</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="0" t="s">
-        <v>690</v>
+        <v>694</v>
       </c>
       <c r="B27" s="0" t="s">
-        <v>691</v>
+        <v>695</v>
       </c>
       <c r="C27" s="0" t="s">
-        <v>619</v>
+        <v>623</v>
       </c>
       <c r="D27" s="0" t="s">
-        <v>692</v>
+        <v>696</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="0" t="s">
-        <v>693</v>
+        <v>697</v>
       </c>
       <c r="B28" s="0" t="s">
-        <v>694</v>
+        <v>698</v>
       </c>
       <c r="C28" s="0" t="s">
-        <v>619</v>
+        <v>623</v>
       </c>
       <c r="D28" s="0" t="s">
-        <v>695</v>
+        <v>699</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="0" t="s">
-        <v>696</v>
+        <v>700</v>
       </c>
       <c r="B29" s="0" t="s">
-        <v>697</v>
+        <v>701</v>
       </c>
       <c r="C29" s="0" t="s">
-        <v>619</v>
+        <v>623</v>
       </c>
       <c r="D29" s="0" t="s">
-        <v>698</v>
+        <v>702</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="0" t="s">
-        <v>699</v>
+        <v>703</v>
       </c>
       <c r="B30" s="0" t="s">
-        <v>700</v>
+        <v>704</v>
       </c>
       <c r="C30" s="0" t="s">
-        <v>439</v>
+        <v>443</v>
       </c>
       <c r="D30" s="0" t="s">
-        <v>701</v>
+        <v>705</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="0" t="s">
-        <v>702</v>
+        <v>706</v>
       </c>
       <c r="B31" s="0" t="s">
-        <v>703</v>
+        <v>707</v>
       </c>
       <c r="C31" s="0" t="s">
-        <v>619</v>
+        <v>623</v>
       </c>
       <c r="D31" s="0" t="s">
-        <v>704</v>
+        <v>708</v>
       </c>
     </row>
   </sheetData>
@@ -8616,12 +8694,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="0" t="s">
-        <v>705</v>
+        <v>709</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="0" t="s">
-        <v>706</v>
+        <v>710</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
B&N rev8 WIP: Tek screws #10-16 per 8.A + 7/A-210 runner track Teks (10,132)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01UQBQT8jCVU6KW8QmKhZS83
</commit_message>
<xml_diff>
--- a/cache_proyectos/barnes_noble/takeoff_work/etapas/8_excel/Barnes_Noble_ColoradoSprings_Takeoff_FINAL_rev8.xlsx
+++ b/cache_proyectos/barnes_noble/takeoff_work/etapas/8_excel/Barnes_Noble_ColoradoSprings_Takeoff_FINAL_rev8.xlsx
@@ -1153,10 +1153,10 @@
     <t xml:space="preserve">N/SHEET: 8/A-410 | Breakdown [DERIVED]: PAN-HEAD-8-A410 291 = 291 PCS | 8/A-410 "CONTINUOUS 20 GA. X 2" MIN DEEP RELIEF CHANNEL - ANCHOR TO STEEL PLATE WITH #8 PAN HEAD SELF TAPPING SCREWS AT 24" O.C. AND 6" FROM ENDS": sum(ROUNDUP(L / 2) + 1) over 32 runs to structure (479.85 LF) = 291 pcs (rev7 plan check C7-03; note 8.C X-EDNI = alternative in RFI-51)</t>
   </si>
   <si>
-    <t xml:space="preserve">#8 Tek screws at clip angles ((4) per clip, 5/A-410; 7/A-210)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">N/SHEET: 5/A-410, 7/A-210 | Breakdown [DERIVED]: TEK-SCREWS-CLIPS 10,088 = 10,088 PCS | 5/A-410 "2" x 2" 16 GA. CLIP ANGLE ... (4) TEK SCREWS": 2518 clips x 4 = 10072 + 7/A-210 "(4) #10-16 SCREWS": 4 clips x 4 = 16; total 10088 pcs</t>
+    <t xml:space="preserve">#10-16 x 3/4" Tek screws, pan head, at 16 ga clip angles and nested header runner tracks (5/A-410; 7/A-210; A-410 note 8.A)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">N/SHEET: 5/A-410, 7/A-210 | Breakdown [DERIVED]: TEK-SCREWS-CLIPS 10,132 = 10,132 PCS | 5/A-410 "2" x 2" 16 GA. CLIP ANGLE ... (4) TEK SCREWS": 2518 clips x 4 = 10072 + 7/A-210 "(4) #10-16 SCREWS": 4 clips x 4 = 16 + 7/A-210 "RUNNER TRACK ATTACHED TO HEADER SUING (2) TEK SCREWS AT 16" O.C" top and bottom runner: 2 runners x 2 x (ROUNDUP(12.667 / 1.333) + 1) = 44; total 10132 pcs. Size: 5/A-410 prints none; the clip is 16 ga, so A-410 note 8.A "18/16 GAUGE - #10 - 16 X 3/4" TEKS" applies (7/A-210 prints #10-16)</t>
   </si>
   <si>
     <t xml:space="preserve">16 ga wire at seismic brace points (5/A-121)</t>
@@ -2158,7 +2158,7 @@
     <t xml:space="preserve">reglas.py compuerta OK</t>
   </si>
   <si>
-    <t xml:space="preserve">{"canon": "10f5767fbe6d10175f7550f9277cd486c29266b3548a6196084574efbcbdf683", "evidencias": "82f4ec13c901d7191f9772989e98854d158340ab19499f6cfbada96ca6cbd21e", "familias_out": "5e80b25c4c58f2a7c1ce346a2e981b61dd297fac8c01d5924de335dd8fefe16b", "reglas": "e6de403e47b5aff83e6ca5064f657f448b59ec1e6bbfaf2c2faf6ce87f8729ce", "version": "v73"}</t>
+    <t xml:space="preserve">{"canon": "e23ca4ed4ba05bbad3579c9a6fb335ea586404f3c3e957079d75dd810f51b4f6", "evidencias": "82f4ec13c901d7191f9772989e98854d158340ab19499f6cfbada96ca6cbd21e", "familias_out": "be72b10dead2fcaf2b9134c90ad0d4b77a168739333a4260499f86aac18db698", "reglas": "e6de403e47b5aff83e6ca5064f657f448b59ec1e6bbfaf2c2faf6ce87f8729ce", "version": "v73"}</t>
   </si>
 </sst>
 </file>
@@ -6467,7 +6467,7 @@
         <v>371</v>
       </c>
       <c r="C28" s="0" t="n">
-        <v>10088</v>
+        <v>10132</v>
       </c>
       <c r="D28" s="0" t="n">
         <f aca="false">Inputs!$B$5</f>
@@ -6475,18 +6475,18 @@
       </c>
       <c r="E28" s="0" t="n">
         <f aca="false">C28*D28</f>
-        <v>1513.2</v>
+        <v>1519.8</v>
       </c>
       <c r="F28" s="0" t="n">
         <f aca="false">C28+E28</f>
-        <v>11601.2</v>
+        <v>11651.8</v>
       </c>
       <c r="G28" s="0" t="s">
         <v>355</v>
       </c>
       <c r="H28" s="0" t="n">
         <f aca="false">ROUNDUP(F28,0)</f>
-        <v>11602</v>
+        <v>11652</v>
       </c>
       <c r="I28" s="0" t="s">
         <v>376</v>

</xml_diff>

<commit_message>
B&N rev8 WIP: 8/A-210 nested column/beam Teks + 7/A-210 head attachment (Tek row 10,668), RFI-51 delta
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01UQBQT8jCVU6KW8QmKhZS83
</commit_message>
<xml_diff>
--- a/cache_proyectos/barnes_noble/takeoff_work/etapas/8_excel/Barnes_Noble_ColoradoSprings_Takeoff_FINAL_rev8.xlsx
+++ b/cache_proyectos/barnes_noble/takeoff_work/etapas/8_excel/Barnes_Noble_ColoradoSprings_Takeoff_FINAL_rev8.xlsx
@@ -1153,10 +1153,10 @@
     <t xml:space="preserve">N/SHEET: 8/A-410 | Breakdown [DERIVED]: PAN-HEAD-8-A410 291 = 291 PCS | 8/A-410 "CONTINUOUS 20 GA. X 2" MIN DEEP RELIEF CHANNEL - ANCHOR TO STEEL PLATE WITH #8 PAN HEAD SELF TAPPING SCREWS AT 24" O.C. AND 6" FROM ENDS": sum(ROUNDUP(L / 2) + 1) over 32 runs to structure (479.85 LF) = 291 pcs (rev7 plan check C7-03; note 8.C X-EDNI = alternative in RFI-51)</t>
   </si>
   <si>
-    <t xml:space="preserve">#10-16 x 3/4" Tek screws, pan head, at 16 ga clip angles and nested header runner tracks (5/A-410; 7/A-210; A-410 note 8.A)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">N/SHEET: 5/A-410, 7/A-210 | Breakdown [DERIVED]: TEK-SCREWS-CLIPS 10,132 = 10,132 PCS | 5/A-410 "2" x 2" 16 GA. CLIP ANGLE ... (4) TEK SCREWS": 2518 clips x 4 = 10072 + 7/A-210 "(4) #10-16 SCREWS": 4 clips x 4 = 16 + 7/A-210 "RUNNER TRACK ATTACHED TO HEADER SUING (2) TEK SCREWS AT 16" O.C" top and bottom runner: 2 runners x 2 x (ROUNDUP(12.667 / 1.333) + 1) = 44; total 10132 pcs. Size: 5/A-410 prints none; the clip is 16 ga, so A-410 note 8.A "18/16 GAUGE - #10 - 16 X 3/4" TEKS" applies (7/A-210 prints #10-16)</t>
+    <t xml:space="preserve">#10-16 x 3/4" Tek screws, pan head, at 16 ga clip angles and nested header / column / beam (5/A-410; 7/A-210; 8/A-210; A-410 note 8.A)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">N/SHEET: 5/A-410, 7/A-210, 8/A-210, 1/A-210 | Breakdown [DERIVED]: TEK-SCREWS-CLIPS 10,668 = 10,668 PCS | 5/A-410 "2" x 2" 16 GA. CLIP ANGLE ... (4) TEK SCREWS": 2518 clips x 4 = 10072 + 7/A-210 "(4) #10-16 SCREWS": 4 clips x 4 = 16 + 7/A-210 "RUNNER TRACK ATTACHED TO HEADER SUING (2) TEK SCREWS AT 16" O.C" top and bottom runner: 2 runners x 2 x (ROUNDUP(12.667 / 1.333) + 1) = 44 + 8/A-210 "(8) #10-16 TEKS 16"O.C., TYP.": nested beam (ROUNDUP(12.667 / 1.333) + 1) x 8 = 88 + nested columns 6 x (ROUNDUP(10.5 / 1.333) + 1) x 8 = 432 + 7/A-210 head attachment "#10-16 TEK SCREWS (TYP.)": 2 clips x 8 = 16; total 10668 pcs. Header 12'-8" = 1/A-210 front dimension chain (152"). Size: 5/A-410 prints none; the clip is 16 ga, so A-410 note 8.A "18/16 GAUGE - #10 - 16 X 3/4" TEKS" applies (7/A-210 and 8/A-210 print #10-16)</t>
   </si>
   <si>
     <t xml:space="preserve">16 ga wire at seismic brace points (5/A-121)</t>
@@ -1846,7 +1846,7 @@
     <t xml:space="preserve">Fastener counts not printed: 7/A-210 3"x3"x16 ga clip angles (count per header end); cement board screw spacing (manufacturer standard 8" O.C. used); plywood screws per A-410 note 8.D (24" field / 12" perimeter on 4x8 sheets).</t>
   </si>
   <si>
-    <t xml:space="preserve">Carried: clip angles 7/A-210 4 pcs; cement board screws 1686 pcs; plywood screws 2331 pcs - adjust to the estimator yields. Framing screws count the stud pieces of the walls and column wraps (781); the detail members (braces, cross members, bracing) add about + 724 screws. 9/A-410 calls #8 screws stud to track while note 8.A calls #10-16 on 18/16 ga - carried per 8.A. Plan check (rev8): relief channel to structure carried with 8/A-410 #8 pan head screws (291 pcs) + P.A.F. at cross members (282 pcs); note 8.C X-EDNI (2 rows @ 16" = 720 pcs) is the alternative if the track bears directly on structural steel. Slab pins carried per note 8.F (2 rows @ 16" X-DNI); 9/A-410 alternative 0.177" PAF @ 24" = - 640.61 pcs.</t>
+    <t xml:space="preserve">Carried: clip angles 7/A-210 4 pcs; cement board screws 1686 pcs; plywood screws 2331 pcs - adjust to the estimator yields. Framing screws count the stud pieces of the walls and column wraps (781); the detail members (braces, cross members, bracing) add about + 724 screws. 9/A-410 calls #8 screws stud to track while note 8.A calls #10-16 on 18/16 ga - carried per 8.A. Plan check (rev8): relief channel to structure carried with 8/A-410 #8 pan head screws (291 pcs) + P.A.F. at cross members (282 pcs); note 8.C X-EDNI (2 rows @ 16" = 720 pcs) is the alternative if the track bears directly on structural steel. Slab pins carried per note 8.F (2 rows @ 16" X-DNI); 9/A-410 alternative 0.177" PAF @ 24" = - 640.61 pcs. 8/A-210 "(8) #10-16 TEKS 16"O.C., TYP." read as 8 per station at 16" O.C. (520 pcs carried); if 8 per member in total: - 464 pcs. 7/A-210 head attachment clips: 2 assumed (16 screws), count not printed.</t>
   </si>
   <si>
     <t xml:space="preserve">0 questions in total, asked ONE at a time in this order: floor plan (partition types A-Z), then the details the floor plan calls, in order</t>
@@ -2158,7 +2158,7 @@
     <t xml:space="preserve">reglas.py compuerta OK</t>
   </si>
   <si>
-    <t xml:space="preserve">{"canon": "e23ca4ed4ba05bbad3579c9a6fb335ea586404f3c3e957079d75dd810f51b4f6", "evidencias": "82f4ec13c901d7191f9772989e98854d158340ab19499f6cfbada96ca6cbd21e", "familias_out": "be72b10dead2fcaf2b9134c90ad0d4b77a168739333a4260499f86aac18db698", "reglas": "e6de403e47b5aff83e6ca5064f657f448b59ec1e6bbfaf2c2faf6ce87f8729ce", "version": "v73"}</t>
+    <t xml:space="preserve">{"canon": "4d10543c89c7c875c17b966c097706428d9afc8b032d68cbb8cd59e20a8894c7", "evidencias": "82f4ec13c901d7191f9772989e98854d158340ab19499f6cfbada96ca6cbd21e", "familias_out": "3903f0f0348356f461af86dc2e592a30917780abcfdddef5c5eb885ad68849e4", "reglas": "e6de403e47b5aff83e6ca5064f657f448b59ec1e6bbfaf2c2faf6ce87f8729ce", "version": "v73"}</t>
   </si>
 </sst>
 </file>
@@ -6467,7 +6467,7 @@
         <v>371</v>
       </c>
       <c r="C28" s="0" t="n">
-        <v>10132</v>
+        <v>10668</v>
       </c>
       <c r="D28" s="0" t="n">
         <f aca="false">Inputs!$B$5</f>
@@ -6475,18 +6475,18 @@
       </c>
       <c r="E28" s="0" t="n">
         <f aca="false">C28*D28</f>
-        <v>1519.8</v>
+        <v>1600.2</v>
       </c>
       <c r="F28" s="0" t="n">
         <f aca="false">C28+E28</f>
-        <v>11651.8</v>
+        <v>12268.2</v>
       </c>
       <c r="G28" s="0" t="s">
         <v>355</v>
       </c>
       <c r="H28" s="0" t="n">
         <f aca="false">ROUNDUP(F28,0)</f>
-        <v>11652</v>
+        <v>12269</v>
       </c>
       <c r="I28" s="0" t="s">
         <v>376</v>

</xml_diff>